<commit_message>
Freeze Revision D.1 release evidence and manifest
</commit_message>
<xml_diff>
--- a/10_schedules/FC01_engineering_schedules.xlsx
+++ b/10_schedules/FC01_engineering_schedules.xlsx
@@ -19911,7 +19911,7 @@
         <x:v>VAL-D-STATIC</x:v>
       </x:c>
       <x:c r="G24" s="6" t="str">
-        <x:v>Revision-D canonical/source/schedule validation suite; the executed report records the current check count</x:v>
+        <x:v>Revision-D.1 canonical/source/schedule validation suite; the executed report records the current check count</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="54" customHeight="1">
@@ -21109,7 +21109,7 @@
         <x:v>Electrical owner</x:v>
       </x:c>
       <x:c r="D20" s="6" t="str">
-        <x:v>Revision-D FCStd/exchange validation</x:v>
+        <x:v>Revision-D.1 FCStd/exchange validation</x:v>
       </x:c>
       <x:c r="E20" s="6" t="str">
         <x:v>OPEN</x:v>
@@ -21155,7 +21155,7 @@
         <x:v>Electrical owner</x:v>
       </x:c>
       <x:c r="D22" s="6" t="str">
-        <x:v>Revision-D schematic authoring, reopen, export and review</x:v>
+        <x:v>Revision-D.1 schematic authoring, reopen, export and review</x:v>
       </x:c>
       <x:c r="E22" s="6" t="str">
         <x:v>OPEN</x:v>
@@ -21362,7 +21362,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Revision-D deterministic validator and source-parity checks pass; see current automated report for count</x:v>
+        <x:v>Revision-D.1 deterministic validator and source-parity checks pass; see current automated report for count</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="54" customHeight="1">
@@ -21468,7 +21468,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
-        <x:v>Revision-D QET reopens and reconciles</x:v>
+        <x:v>Revision-D.1 QET reopens and reconciles</x:v>
       </x:c>
       <x:c r="C11" s="6" t="str">
         <x:v>BLOCKED</x:v>
@@ -21488,7 +21488,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D12" s="6" t="str">
-        <x:v>Revision-D native schematics do not exist</x:v>
+        <x:v>Revision-D.1 native schematics do not exist</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
@@ -21496,7 +21496,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="6" t="str">
-        <x:v>Revision-D FCStd reopens</x:v>
+        <x:v>Revision-D.1 FCStd reopens</x:v>
       </x:c>
       <x:c r="C13" s="6" t="str">
         <x:v>BLOCKED</x:v>
@@ -21516,7 +21516,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D14" s="6" t="str">
-        <x:v>Revision-D exchange files do not exist and FreeCAD is absent</x:v>
+        <x:v>Revision-D.1 exchange files do not exist and FreeCAD is absent</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
@@ -21600,7 +21600,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D20" s="6" t="str">
-        <x:v>Local source-design scope: simulator, 32 scenarios, edge service, interface harness and Revision-D independent interface-oracle tests pass; native integration remains blocked under gates 9 and 18</x:v>
+        <x:v>Local source-design scope: simulator, 32 scenarios, edge service, interface harness and Revision-D.1 independent interface-oracle tests pass; native integration remains blocked under gates 9 and 18</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
@@ -23888,7 +23888,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="24" t="str">
-        <x:v>FICTIONAL ENGINEERING PROJECT — NOT FOR CONSTRUCTION | Revision D | Professional controlled engineering-development package</x:v>
+        <x:v>FICTIONAL ENGINEERING PROJECT — NOT FOR CONSTRUCTION | Revision D.1 | Professional controlled engineering-development release candidate</x:v>
       </x:c>
       <x:c r="B3" s="24"/>
       <x:c r="C3" s="24"/>
@@ -23934,7 +23934,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="D6" s="46" t="str">
-        <x:v>Native TIA/WinCC/Startdrive/PLCSIM, trained NVIDIA model, Revision-D QElectroTech and Revision-D panel CAD remain blocked. Historical native electrical/CAD files are quarantined baselines. No construction, safety, native compile, FAT, SAT or model-performance claim is made.</x:v>
+        <x:v>Native TIA/WinCC/Startdrive/PLCSIM, trained NVIDIA model, Revision-D.1 QElectroTech and Revision-D.1 panel CAD remain blocked. Historical native electrical/CAD files are byte-exact quarantined baselines. No construction, safety, native compile, FAT, SAT or model-performance claim is made.</x:v>
       </x:c>
       <x:c r="E6" s="46"/>
       <x:c r="F6" s="46"/>

</xml_diff>

<commit_message>
feat: execute Revision E native engineering
</commit_message>
<xml_diff>
--- a/10_schedules/FC01_engineering_schedules.xlsx
+++ b/10_schedules/FC01_engineering_schedules.xlsx
@@ -21,7 +21,8 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Coverage" sheetId="17" r:id="rId20"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input Requests" sheetId="18" r:id="rId21"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Gates" sheetId="19" r:id="rId22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Summary" sheetId="20" r:id="rId23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document Register" sheetId="20" r:id="rId23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Summary" sheetId="21" r:id="rId24"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -461,6 +462,21 @@
 </x:table>
 </file>
 
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="DocumentRegisterTable" displayName="DocumentRegisterTable" ref="A1:F14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F14"/>
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="document_id"/>
+    <x:tableColumn id="2" name="title"/>
+    <x:tableColumn id="3" name="path"/>
+    <x:tableColumn id="4" name="revision"/>
+    <x:tableColumn id="5" name="owner"/>
+    <x:tableColumn id="6" name="status"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DrivePZDTable" displayName="DrivePZDTable" ref="A1:J9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:J9"/>
@@ -1151,11 +1167,17 @@
       <x:c r="H8" s="6" t="str">
         <x:v>Startdrive selection open</x:v>
       </x:c>
-      <x:c r="I8" s="6" t="str"/>
-      <x:c r="J8" s="6" t="str"/>
-      <x:c r="K8" s="6" t="str"/>
+      <x:c r="I8" s="6" t="str">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="str">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="K8" s="6" t="str">
+        <x:v>225.4</x:v>
+      </x:c>
       <x:c r="L8" s="6" t="str">
-        <x:v>Rating, envelope and clearances blocked by motor/mechanics and native Startdrive</x:v>
+        <x:v>SELECTED ENVELOPE; drive rating/duty and Startdrive configuration remain provisional</x:v>
       </x:c>
       <x:c r="M8" s="6" t="str">
         <x:v>https://mall.industry.siemens.com/mall/en/WW/Catalog/Product/6SL3210-1KE12-3UF2</x:v>
@@ -1192,11 +1214,17 @@
       <x:c r="H9" s="6" t="str">
         <x:v>Startdrive selection open</x:v>
       </x:c>
-      <x:c r="I9" s="6" t="str"/>
-      <x:c r="J9" s="6" t="str"/>
-      <x:c r="K9" s="6" t="str"/>
+      <x:c r="I9" s="6" t="str">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="J9" s="6" t="str">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="K9" s="6" t="str">
+        <x:v>225.4</x:v>
+      </x:c>
       <x:c r="L9" s="6" t="str">
-        <x:v>Rating, envelope and clearances blocked by pump curve and motor data</x:v>
+        <x:v>SELECTED ENVELOPE; drive rating/duty and Startdrive configuration remain provisional</x:v>
       </x:c>
       <x:c r="M9" s="6" t="str">
         <x:v>https://mall.industry.siemens.com/mall/en/WW/Catalog/Product/6SL3210-1KE12-3UF2</x:v>
@@ -1280,7 +1308,9 @@
       <x:c r="H11" s="6" t="str">
         <x:v>Native configuration open</x:v>
       </x:c>
-      <x:c r="I11" s="6" t="str"/>
+      <x:c r="I11" s="6" t="str">
+        <x:v>35</x:v>
+      </x:c>
       <x:c r="J11" s="6" t="str">
         <x:v>147</x:v>
       </x:c>
@@ -1288,7 +1318,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="L11" s="6" t="str">
-        <x:v>Exact width and site policy remain procurement/native gates</x:v>
+        <x:v>SELECTED NETWORK BASELINE — native configuration and site policy open</x:v>
       </x:c>
       <x:c r="M11" s="6" t="str">
         <x:v>https://mall.industry.siemens.com/mall/en/oeii/Catalog/Product?SiepCountryCode=OE&amp;mlfb=6GK5615-0AA01-2AA2</x:v>
@@ -1323,11 +1353,17 @@
       <x:c r="H12" s="6" t="str">
         <x:v>JetPack/DeepStream image not selected</x:v>
       </x:c>
-      <x:c r="I12" s="6" t="str"/>
-      <x:c r="J12" s="6" t="str"/>
-      <x:c r="K12" s="6" t="str"/>
+      <x:c r="I12" s="6" t="str">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="J12" s="6" t="str">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="K12" s="6" t="str">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="L12" s="6" t="str">
-        <x:v>Carrier, thermals, power, EMC and lifecycle are open</x:v>
+        <x:v>TBD — NOT PROCUREMENT OR CONSTRUCTION DATA; confirm industrial carrier, thermal solution, EMC and lifecycle</x:v>
       </x:c>
       <x:c r="M12" s="6" t="str">
         <x:v>https://developer.nvidia.com/deepstream-sdk</x:v>
@@ -18666,10 +18702,10 @@
         <x:v>-A100</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>120</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>90</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>35</x:v>
@@ -18687,7 +18723,7 @@
         <x:v>Vertical unless manufacturer requires otherwise</x:v>
       </x:c>
       <x:c r="I2" s="6" t="str">
-        <x:v>Controls</x:v>
+        <x:v>PLC / control</x:v>
       </x:c>
       <x:c r="J2" s="6" t="str">
         <x:v>25</x:v>
@@ -18696,16 +18732,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="L2" s="6" t="str">
-        <x:v>15</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M2" s="6" t="str">
-        <x:v>Manufacturer data required</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="N2" s="6" t="str">
-        <x:v>Official Siemens data sheet</x:v>
+        <x:v>Official Siemens product data; simplified rectangular selected-device envelope</x:v>
       </x:c>
       <x:c r="O2" s="6" t="str">
-        <x:v>Coordinate reserved; native CAD and clearance verification open</x:v>
+        <x:v>SELECTED BASELINE — native TIA catalog/configuration and accessory confirmation open</x:v>
       </x:c>
       <x:c r="P2" s="6" t="str">
         <x:v>=FC01+CP01-A100</x:v>
@@ -18716,10 +18752,10 @@
         <x:v>-A101</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>185</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>90</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
         <x:v>35</x:v>
@@ -18737,7 +18773,7 @@
         <x:v>Vertical unless manufacturer requires otherwise</x:v>
       </x:c>
       <x:c r="I3" s="6" t="str">
-        <x:v>Controls</x:v>
+        <x:v>PLC / control</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
         <x:v>25</x:v>
@@ -18746,16 +18782,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="L3" s="6" t="str">
-        <x:v>15</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M3" s="6" t="str">
-        <x:v>Manufacturer data required</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="N3" s="6" t="str">
-        <x:v>Official Siemens data sheet</x:v>
+        <x:v>Official Siemens product data; simplified rectangular selected-device envelope</x:v>
       </x:c>
       <x:c r="O3" s="6" t="str">
-        <x:v>Coordinate reserved; native CAD and clearance verification open</x:v>
+        <x:v>SELECTED BASELINE — native TIA catalog/configuration and accessory confirmation open</x:v>
       </x:c>
       <x:c r="P3" s="6" t="str">
         <x:v>=FC01+CP01-A101</x:v>
@@ -18766,10 +18802,10 @@
         <x:v>-A102</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>250</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>90</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
         <x:v>35</x:v>
@@ -18787,7 +18823,7 @@
         <x:v>Vertical unless manufacturer requires otherwise</x:v>
       </x:c>
       <x:c r="I4" s="6" t="str">
-        <x:v>Controls</x:v>
+        <x:v>PLC / control</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
         <x:v>25</x:v>
@@ -18796,16 +18832,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="L4" s="6" t="str">
-        <x:v>15</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M4" s="6" t="str">
-        <x:v>Manufacturer data required</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="N4" s="6" t="str">
-        <x:v>Official Siemens data sheet</x:v>
+        <x:v>Official Siemens product data; simplified rectangular selected-device envelope</x:v>
       </x:c>
       <x:c r="O4" s="6" t="str">
-        <x:v>Coordinate reserved; native CAD and clearance verification open</x:v>
+        <x:v>SELECTED BASELINE — native TIA catalog/configuration and accessory confirmation open</x:v>
       </x:c>
       <x:c r="P4" s="6" t="str">
         <x:v>=FC01+CP01-A102</x:v>
@@ -18816,10 +18852,10 @@
         <x:v>-A103</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
-        <x:v>315</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="C5" s="6" t="str">
-        <x:v>90</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="D5" s="6" t="str">
         <x:v>35</x:v>
@@ -18837,7 +18873,7 @@
         <x:v>Vertical unless manufacturer requires otherwise</x:v>
       </x:c>
       <x:c r="I5" s="6" t="str">
-        <x:v>Controls</x:v>
+        <x:v>PLC / control</x:v>
       </x:c>
       <x:c r="J5" s="6" t="str">
         <x:v>25</x:v>
@@ -18846,16 +18882,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="L5" s="6" t="str">
-        <x:v>15</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M5" s="6" t="str">
-        <x:v>Manufacturer data required</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="N5" s="6" t="str">
-        <x:v>Official Siemens data sheet</x:v>
+        <x:v>Official Siemens product data; simplified rectangular selected-device envelope</x:v>
       </x:c>
       <x:c r="O5" s="6" t="str">
-        <x:v>Coordinate reserved; native CAD and clearance verification open</x:v>
+        <x:v>SELECTED BASELINE — native TIA catalog/configuration and accessory confirmation open</x:v>
       </x:c>
       <x:c r="P5" s="6" t="str">
         <x:v>=FC01+CP01-A103</x:v>
@@ -18866,10 +18902,10 @@
         <x:v>-A104</x:v>
       </x:c>
       <x:c r="B6" s="6" t="str">
-        <x:v>380</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="C6" s="6" t="str">
-        <x:v>90</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="D6" s="6" t="str">
         <x:v>35</x:v>
@@ -18887,7 +18923,7 @@
         <x:v>Vertical unless manufacturer requires otherwise</x:v>
       </x:c>
       <x:c r="I6" s="6" t="str">
-        <x:v>Analog</x:v>
+        <x:v>PLC / control</x:v>
       </x:c>
       <x:c r="J6" s="6" t="str">
         <x:v>25</x:v>
@@ -18896,16 +18932,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="L6" s="6" t="str">
-        <x:v>15</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M6" s="6" t="str">
-        <x:v>Manufacturer data required</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="N6" s="6" t="str">
-        <x:v>Official Siemens data sheet</x:v>
+        <x:v>Official Siemens product data; simplified rectangular selected-device envelope</x:v>
       </x:c>
       <x:c r="O6" s="6" t="str">
-        <x:v>Coordinate reserved; native CAD and clearance verification open</x:v>
+        <x:v>SELECTED BASELINE — native TIA catalog/configuration and accessory confirmation open</x:v>
       </x:c>
       <x:c r="P6" s="6" t="str">
         <x:v>=FC01+CP01-A104</x:v>
@@ -18916,19 +18952,19 @@
         <x:v>-H100</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
-        <x:v>290</x:v>
+        <x:v>300.85</x:v>
       </x:c>
       <x:c r="C7" s="6" t="str">
-        <x:v>200</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="D7" s="6" t="str">
-        <x:v>214</x:v>
+        <x:v>198.3</x:v>
       </x:c>
       <x:c r="E7" s="6" t="str">
-        <x:v>158</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="F7" s="6" t="str">
-        <x:v>63.6</x:v>
+        <x:v>55.6</x:v>
       </x:c>
       <x:c r="G7" s="6" t="str">
         <x:v>Door cutout</x:v>
@@ -18940,22 +18976,22 @@
         <x:v>HMI</x:v>
       </x:c>
       <x:c r="J7" s="6" t="str">
-        <x:v>25</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K7" s="6" t="str">
-        <x:v>25</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L7" s="6" t="str">
-        <x:v>15</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M7" s="6" t="str">
-        <x:v>Manufacturer data required</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="N7" s="6" t="str">
-        <x:v>Official Siemens data sheet</x:v>
+        <x:v>Official Siemens envelope/cutout: outer 214 x 158 x 63.6 mm; cutout 198.3 x 142 mm</x:v>
       </x:c>
       <x:c r="O7" s="6" t="str">
-        <x:v>Coordinate reserved; native CAD and clearance verification open</x:v>
+        <x:v>SELECTED BASELINE — native WinCC project/compile and door reinforcement open</x:v>
       </x:c>
       <x:c r="P7" s="6" t="str">
         <x:v>=FC01+CP01-H100</x:v>
@@ -18966,40 +19002,46 @@
         <x:v>-U100</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
-        <x:v>120</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C8" s="6" t="str">
-        <x:v>430</x:v>
-      </x:c>
-      <x:c r="D8" s="6" t="str"/>
-      <x:c r="E8" s="6" t="str"/>
-      <x:c r="F8" s="6" t="str"/>
+        <x:v>275</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>225.4</x:v>
+      </x:c>
       <x:c r="G8" s="6" t="str">
-        <x:v>Mounting plate</x:v>
+        <x:v>Direct mounting plate</x:v>
       </x:c>
       <x:c r="H8" s="6" t="str">
         <x:v>Vertical unless manufacturer requires otherwise</x:v>
       </x:c>
       <x:c r="I8" s="6" t="str">
-        <x:v>VFD heat zone</x:v>
+        <x:v>Mains / drive heat</x:v>
       </x:c>
       <x:c r="J8" s="6" t="str">
-        <x:v>100</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="K8" s="6" t="str">
         <x:v>100</x:v>
       </x:c>
       <x:c r="L8" s="6" t="str">
-        <x:v>50</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M8" s="6" t="str">
-        <x:v>TBD</x:v>
+        <x:v>38.6</x:v>
       </x:c>
       <x:c r="N8" s="6" t="str">
-        <x:v>OPEN - exact selected-device envelope unavailable</x:v>
+        <x:v>Siemens order-number data sheet: 73 W x 196 H x 225.4 D mm; FSA PN</x:v>
       </x:c>
       <x:c r="O8" s="6" t="str">
-        <x:v>Coordinate reserved; native CAD and clearance verification open</x:v>
+        <x:v>SELECTED ENVELOPE; drive rating/duty and Startdrive configuration remain provisional</x:v>
       </x:c>
       <x:c r="P8" s="6" t="str">
         <x:v>=FC01+CP01-U100</x:v>
@@ -19010,40 +19052,46 @@
         <x:v>-U101</x:v>
       </x:c>
       <x:c r="B9" s="6" t="str">
-        <x:v>370</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="C9" s="6" t="str">
-        <x:v>430</x:v>
-      </x:c>
-      <x:c r="D9" s="6" t="str"/>
-      <x:c r="E9" s="6" t="str"/>
-      <x:c r="F9" s="6" t="str"/>
+        <x:v>275</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="str">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="str">
+        <x:v>225.4</x:v>
+      </x:c>
       <x:c r="G9" s="6" t="str">
-        <x:v>Mounting plate</x:v>
+        <x:v>Direct mounting plate</x:v>
       </x:c>
       <x:c r="H9" s="6" t="str">
         <x:v>Vertical unless manufacturer requires otherwise</x:v>
       </x:c>
       <x:c r="I9" s="6" t="str">
-        <x:v>VFD heat zone</x:v>
+        <x:v>Mains / drive heat</x:v>
       </x:c>
       <x:c r="J9" s="6" t="str">
-        <x:v>100</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="K9" s="6" t="str">
         <x:v>100</x:v>
       </x:c>
       <x:c r="L9" s="6" t="str">
-        <x:v>50</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M9" s="6" t="str">
-        <x:v>TBD</x:v>
+        <x:v>38.6</x:v>
       </x:c>
       <x:c r="N9" s="6" t="str">
-        <x:v>OPEN - exact selected-device envelope unavailable</x:v>
+        <x:v>Siemens order-number data sheet: 73 W x 196 H x 225.4 D mm; FSA PN</x:v>
       </x:c>
       <x:c r="O9" s="6" t="str">
-        <x:v>Coordinate reserved; native CAD and clearance verification open</x:v>
+        <x:v>SELECTED ENVELOPE; drive rating/duty and Startdrive configuration remain provisional</x:v>
       </x:c>
       <x:c r="P9" s="6" t="str">
         <x:v>=FC01+CP01-U101</x:v>
@@ -19054,10 +19102,10 @@
         <x:v>-SW100</x:v>
       </x:c>
       <x:c r="B10" s="6" t="str">
-        <x:v>450</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="C10" s="6" t="str">
-        <x:v>90</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="D10" s="6" t="str">
         <x:v>60</x:v>
@@ -19084,16 +19132,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="L10" s="6" t="str">
-        <x:v>15</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M10" s="6" t="str">
-        <x:v>Manufacturer data required</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="N10" s="6" t="str">
-        <x:v>Official Siemens data sheet</x:v>
+        <x:v>Official Siemens technical data; controlled 5 mm lateral layout-clearance assumption; confirm against order-number installation data</x:v>
       </x:c>
       <x:c r="O10" s="6" t="str">
-        <x:v>Coordinate reserved; native CAD and clearance verification open</x:v>
+        <x:v>SELECTED NETWORK BASELINE — native configuration and site policy open</x:v>
       </x:c>
       <x:c r="P10" s="6" t="str">
         <x:v>=FC01+CP01-SW100</x:v>
@@ -19104,12 +19152,14 @@
         <x:v>-FW100</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
-        <x:v>540</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="C11" s="6" t="str">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="D11" s="6" t="str"/>
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>35</x:v>
+      </x:c>
       <x:c r="E11" s="6" t="str">
         <x:v>147</x:v>
       </x:c>
@@ -19132,16 +19182,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="L11" s="6" t="str">
-        <x:v>15</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M11" s="6" t="str">
-        <x:v>Manufacturer data required</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="N11" s="6" t="str">
-        <x:v>OPEN - exact selected-device envelope unavailable</x:v>
+        <x:v>Siemens S615/S615 EEC operating instructions; variant CAx confirmation open; controlled 5 mm lateral layout-clearance assumption; confirm against order-number installation data</x:v>
       </x:c>
       <x:c r="O11" s="6" t="str">
-        <x:v>Coordinate reserved; native CAD and clearance verification open</x:v>
+        <x:v>SELECTED NETWORK BASELINE — native configuration and site policy open</x:v>
       </x:c>
       <x:c r="P11" s="6" t="str">
         <x:v>=FC01+CP01-FW100</x:v>
@@ -19152,14 +19202,20 @@
         <x:v>-PC200</x:v>
       </x:c>
       <x:c r="B12" s="6" t="str">
-        <x:v>600</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="C12" s="6" t="str">
-        <x:v>250</x:v>
-      </x:c>
-      <x:c r="D12" s="6" t="str"/>
-      <x:c r="E12" s="6" t="str"/>
-      <x:c r="F12" s="6" t="str"/>
+        <x:v>540</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="str">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="G12" s="6" t="str">
         <x:v>DIN rail / shelf</x:v>
       </x:c>
@@ -19167,7 +19223,7 @@
         <x:v>Vertical unless manufacturer requires otherwise</x:v>
       </x:c>
       <x:c r="I12" s="6" t="str">
-        <x:v>Vision</x:v>
+        <x:v>Vision edge</x:v>
       </x:c>
       <x:c r="J12" s="6" t="str">
         <x:v>25</x:v>
@@ -19176,16 +19232,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="L12" s="6" t="str">
-        <x:v>15</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M12" s="6" t="str">
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="N12" s="6" t="str">
-        <x:v>OPEN - exact selected-device envelope unavailable</x:v>
+        <x:v>CONTROLLED ARCHITECTURE-ONLY ENVELOPE ASSUMPTION — carrier, cooling kit and interfaces not selected</x:v>
       </x:c>
       <x:c r="O12" s="6" t="str">
-        <x:v>Coordinate reserved; native CAD and clearance verification open</x:v>
+        <x:v>TBD — NOT PROCUREMENT OR CONSTRUCTION DATA; confirm industrial carrier, thermal solution, EMC and lifecycle</x:v>
       </x:c>
       <x:c r="P12" s="6" t="str">
         <x:v>=FC01+CP01-PC200</x:v>
@@ -19196,19 +19252,19 @@
         <x:v>-PE100</x:v>
       </x:c>
       <x:c r="B13" s="6" t="str">
-        <x:v>120</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C13" s="6" t="str">
-        <x:v>755</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D13" s="6" t="str">
-        <x:v>630</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="E13" s="6" t="str">
-        <x:v>25</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F13" s="6" t="str">
-        <x:v>25</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G13" s="6" t="str">
         <x:v>Mounting plate</x:v>
@@ -19220,22 +19276,22 @@
         <x:v>PE</x:v>
       </x:c>
       <x:c r="J13" s="6" t="str">
-        <x:v>20</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K13" s="6" t="str">
-        <x:v>20</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L13" s="6" t="str">
-        <x:v>20</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M13" s="6" t="str">
-        <x:v>0</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="N13" s="6" t="str">
-        <x:v>Provisional bar envelope</x:v>
+        <x:v>Controlled provisional bar envelope; section and fixing hardware open</x:v>
       </x:c>
       <x:c r="O13" s="6" t="str">
-        <x:v>Final PE sizing open</x:v>
+        <x:v>TBD — PE sizing, bonding points and fault-current basis required</x:v>
       </x:c>
       <x:c r="P13" s="6" t="str">
         <x:v>=FC01+CP01-PE100</x:v>
@@ -19246,19 +19302,19 @@
         <x:v>-X100..-X199</x:v>
       </x:c>
       <x:c r="B14" s="6" t="str">
-        <x:v>120</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C14" s="6" t="str">
-        <x:v>650</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="D14" s="6" t="str">
-        <x:v>630</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="E14" s="6" t="str">
         <x:v>50</x:v>
       </x:c>
       <x:c r="F14" s="6" t="str">
-        <x:v>70</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="G14" s="6" t="str">
         <x:v>DIN rail R4</x:v>
@@ -19270,22 +19326,22 @@
         <x:v>Field termination</x:v>
       </x:c>
       <x:c r="J14" s="6" t="str">
-        <x:v>40</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K14" s="6" t="str">
-        <x:v>30</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L14" s="6" t="str">
-        <x:v>20</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M14" s="6" t="str">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N14" s="6" t="str">
-        <x:v>Reserved terminal-row envelope</x:v>
+        <x:v>Revision-E native schedule: 84 logical terminals plus controlled PE/shield terminal objects</x:v>
       </x:c>
       <x:c r="O14" s="6" t="str">
-        <x:v>Terminal family and count open</x:v>
+        <x:v>NATIVE GEOMETRY VERIFIED; terminal family, bridges, accessories and construction release remain open</x:v>
       </x:c>
       <x:c r="P14" s="6" t="str">
         <x:v>=FC01+CP01-X100..-X199</x:v>
@@ -19296,19 +19352,19 @@
         <x:v>-WD100</x:v>
       </x:c>
       <x:c r="B15" s="6" t="str">
-        <x:v>50</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C15" s="6" t="str">
-        <x:v>50</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="D15" s="6" t="str">
-        <x:v>40</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E15" s="6" t="str">
-        <x:v>540</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="F15" s="6" t="str">
-        <x:v>60</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="G15" s="6" t="str">
         <x:v>Mounting plate</x:v>
@@ -19317,7 +19373,7 @@
         <x:v>Vertical duct</x:v>
       </x:c>
       <x:c r="I15" s="6" t="str">
-        <x:v>24 VDC routing</x:v>
+        <x:v>Routing</x:v>
       </x:c>
       <x:c r="J15" s="6" t="str">
         <x:v>0</x:v>
@@ -19326,16 +19382,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L15" s="6" t="str">
-        <x:v>15</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M15" s="6" t="str">
-        <x:v>0</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="N15" s="6" t="str">
-        <x:v>Provisional routing reserve</x:v>
+        <x:v>Controlled routing envelope; duct family and fill calculation open</x:v>
       </x:c>
       <x:c r="O15" s="6" t="str">
-        <x:v>Duct fill calculation open</x:v>
+        <x:v>PROVISIONAL — VERIFY DUCT FILL, bend radius, conductor count and EMC separation</x:v>
       </x:c>
       <x:c r="P15" s="6" t="str">
         <x:v>=FC01+CP01-WD100</x:v>
@@ -19888,7 +19944,7 @@
         <x:v>TC-001..TC-032</x:v>
       </x:c>
       <x:c r="G23" s="6" t="str">
-        <x:v>32 scenario traces and 20 unit/property tests</x:v>
+        <x:v>32 deterministic scenarios plus 88 source/simulator/native-contract tests, 59 edge-service tests and 15 interface-harness tests; see the executed report</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
@@ -19911,7 +19967,7 @@
         <x:v>VAL-D-STATIC</x:v>
       </x:c>
       <x:c r="G24" s="6" t="str">
-        <x:v>Revision-D.1 canonical/source/schedule validation suite; the executed report records the current check count</x:v>
+        <x:v>Revision-E canonical/source/schedule/native-evidence validator; the executed report records the exact current check count</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="54" customHeight="1">
@@ -21103,22 +21159,22 @@
         <x:v>IR-019</x:v>
       </x:c>
       <x:c r="B20" s="6" t="str">
-        <x:v>FreeCAD installation and qualified panel-CAD reviewer</x:v>
+        <x:v>Qualified panel-CAD reviewer, final vendor envelopes/clearances and construction confirmation</x:v>
       </x:c>
       <x:c r="C20" s="6" t="str">
         <x:v>Electrical owner</x:v>
       </x:c>
       <x:c r="D20" s="6" t="str">
-        <x:v>Revision-D.1 FCStd/exchange validation</x:v>
+        <x:v>Construction release of Revision-E native panel CAD</x:v>
       </x:c>
       <x:c r="E20" s="6" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="F20" s="6" t="str">
         <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="G20" s="6" t="str">
-        <x:v>Approved source document or native evidence</x:v>
+        <x:v>Qualified-human review plus approved vendor/site construction data</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
@@ -21149,22 +21205,22 @@
         <x:v>IR-021</x:v>
       </x:c>
       <x:c r="B22" s="6" t="str">
-        <x:v>Usable QElectroTech installation and qualified electrical schematic reviewer</x:v>
+        <x:v>Native reopen/export/all-page review of corrected QET and qualified electrical schematic reviewer</x:v>
       </x:c>
       <x:c r="C22" s="6" t="str">
         <x:v>Electrical owner</x:v>
       </x:c>
       <x:c r="D22" s="6" t="str">
-        <x:v>Revision-D.1 schematic authoring, reopen, export and review</x:v>
+        <x:v>Native schematic gate and construction review</x:v>
       </x:c>
       <x:c r="E22" s="6" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="F22" s="6" t="str">
         <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="G22" s="6" t="str">
-        <x:v>Approved source document or native evidence</x:v>
+        <x:v>Exact corrected-hash QET reopen, PDF export, cross-reference report and qualified-human review</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -21348,7 +21404,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
-        <x:v>Controlled model and tests present; owner approval absent</x:v>
+        <x:v>Controlled model, native-workstream schedules and tests are traceable; identified requirements-owner approval is absent</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="54" customHeight="1">
@@ -21362,7 +21418,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Revision-D.1 deterministic validator and source-parity checks pass; see current automated report for count</x:v>
+        <x:v>Revision-E deterministic validator and source/schedule/native-evidence contracts pass; see current automated report for exact count</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="54" customHeight="1">
@@ -21376,7 +21432,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>V20/FW4.0 design baseline documented; native catalog and delivered state open</x:v>
+        <x:v>V20/FW4.0 source baseline and selected envelopes documented; authorized native catalog confirmation and delivered-state evidence remain open</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="54" customHeight="1">
@@ -21390,7 +21446,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D5" s="6" t="str">
-        <x:v>No genuine AP20 project created</x:v>
+        <x:v>No genuine AP20 project; active identity is not TIA Engineer/Openness-authorized and V20 entitlement is unproven</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
@@ -21404,7 +21460,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D6" s="6" t="str">
-        <x:v>No genuine ZAP20 archive created</x:v>
+        <x:v>No genuine ZAP20 archive exists; native authorized project creation/restoration was not available</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -21418,7 +21474,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D7" s="6" t="str">
-        <x:v>Static source lint only; native compile not run</x:v>
+        <x:v>67 source/simulator contracts pass at Revision-E authoring time; TIA V20 compile was not run</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
@@ -21432,7 +21488,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D8" s="6" t="str">
-        <x:v>WinCC project not created</x:v>
+        <x:v>WinCC V20 components exist but no authorized/licensed native HMI project or compile is proven</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
@@ -21446,7 +21502,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D9" s="6" t="str">
-        <x:v>Startdrive not installed and motor data absent</x:v>
+        <x:v>Startdrive is not installed; motor, pump and site inputs are also missing</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -21460,7 +21516,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D10" s="6" t="str">
-        <x:v>PLCSIM not installed; Python simulator is independent evidence</x:v>
+        <x:v>PLCSIM/PLCSIM Advanced are not installed; deterministic Python evidence is explicitly independent</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -21468,13 +21524,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
-        <x:v>Revision-D.1 QET reopens and reconciles</x:v>
+        <x:v>Revision-E QET reopens and reconciles</x:v>
       </x:c>
       <x:c r="C11" s="6" t="str">
-        <x:v>BLOCKED</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D11" s="6" t="str">
-        <x:v>No runnable QElectroTech found; historical revision-A native baseline only</x:v>
+        <x:v>Corrected 26-folio QET source BCA022BE0B9F65AA061F9731C1EE0BD0399947F04C94EE596D4AD231BB47AAD5 passes 24/24 static and 6/6 contract checks; exact corrected hash was not natively reopened/exported, so native reconciliation remains partial</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -21482,13 +21538,13 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="6" t="str">
-        <x:v>Schematics visual review</x:v>
+        <x:v>Schematics export and all-page visual review</x:v>
       </x:c>
       <x:c r="C12" s="6" t="str">
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D12" s="6" t="str">
-        <x:v>Revision-D.1 native schematics do not exist</x:v>
+        <x:v>Native QET PDF export was not completed and only sampled folios were inspected; all-page visual and native cross-reference review remain blocked</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
@@ -21496,13 +21552,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="6" t="str">
-        <x:v>Revision-D.1 FCStd reopens</x:v>
+        <x:v>Revision-E FCStd reopens</x:v>
       </x:c>
       <x:c r="C13" s="6" t="str">
-        <x:v>BLOCKED</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="D13" s="6" t="str">
-        <x:v>No runnable FreeCAD found; historical baseline only</x:v>
+        <x:v>FreeCADCmd independently reopened 165 objects / 148 controlled solids; STEP retained 148 solids; IGES retained bounded face geometry; DXF entities and 30 scheduled holes reconciled</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="54" customHeight="1">
@@ -21513,10 +21569,10 @@
         <x:v>STEP/IGES/DXF reimport</x:v>
       </x:c>
       <x:c r="C14" s="6" t="str">
-        <x:v>BLOCKED</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="D14" s="6" t="str">
-        <x:v>Revision-D.1 exchange files do not exist and FreeCAD is absent</x:v>
+        <x:v>FreeCADCmd independently reopened 165 objects / 148 controlled solids; STEP retained 148 solids; IGES retained bounded face geometry; DXF entities and 30 scheduled holes reconciled</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
@@ -21530,7 +21586,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D15" s="6" t="str">
-        <x:v>Expanded controlled schedules; unresolved selections and native CAD remain open</x:v>
+        <x:v>Revision-E native layout covers selected architecture and controlled provisional envelopes; final carrier, terminal/relay families, vendor clearances, thermal and construction inputs remain open</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
@@ -21544,7 +21600,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D16" s="6" t="str">
-        <x:v>Site supply, fault current, loads and environmental inputs missing</x:v>
+        <x:v>Supply, earthing, fault current, motors/pump, cable routes, installation method, ambient and enclosure/site requirements remain unconfirmed</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
@@ -21558,7 +21614,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D17" s="6" t="str">
-        <x:v>No real dataset supplied</x:v>
+        <x:v>No representative labeled project dataset or golden/negative image sets were supplied</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
@@ -21572,7 +21628,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D18" s="6" t="str">
-        <x:v>No dataset or TAO runtime</x:v>
+        <x:v>No controlled dataset, training run, evaluated model, ONNX export or defensible metrics exist</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
@@ -21586,7 +21642,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D19" s="6" t="str">
-        <x:v>No selected target carrier/runtime</x:v>
+        <x:v>No selected industrial Jetson carrier/runtime image; CUDA Toolkit, TensorRT, DeepStream and TAO are absent locally</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
@@ -21600,7 +21656,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D20" s="6" t="str">
-        <x:v>Local source-design scope: simulator, 32 scenarios, edge service, interface harness and Revision-D.1 independent interface-oracle tests pass; native integration remains blocked under gates 9 and 18</x:v>
+        <x:v>Source/simulator, edge-service, interface-harness and real asyncua encrypted server/client integration tests pass; production PLC/Jetson endpoint validation remains outside this local gate</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
@@ -21614,7 +21670,7 @@
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="D21" s="6" t="str">
-        <x:v>Procedures issued, never executed</x:v>
+        <x:v>Controlled procedures issued; no FAT, SAT or commissioning was executed</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="54" customHeight="1">
@@ -21628,7 +21684,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D22" s="6" t="str">
-        <x:v>External qualified work required</x:v>
+        <x:v>Project-specific qualified machinery-safety engineering, verification and validation are external and not performed</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -21639,10 +21695,10 @@
         <x:v>Manifest independently verifies</x:v>
       </x:c>
       <x:c r="C23" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D23" s="6" t="str">
-        <x:v>Final deterministic JSON/CSV verifier reports zero missing, unlisted or mismatched files on the frozen release tree; regenerate after any file change</x:v>
+        <x:v>Pre-publication source and generated-artifact controls are implemented; final staged/HEAD manifest, upstream alignment and pushed-commit fresh-clone verification remain pending until the candidate is committed and published</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23855,6 +23911,306 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="10.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22.5" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="31.5" customHeight="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>document_id</x:v>
+      </x:c>
+      <x:c r="B1" s="12" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="C1" s="12" t="str">
+        <x:v>path</x:v>
+      </x:c>
+      <x:c r="D1" s="12" t="str">
+        <x:v>revision</x:v>
+      </x:c>
+      <x:c r="E1" s="12" t="str">
+        <x:v>owner</x:v>
+      </x:c>
+      <x:c r="F1" s="12" t="str">
+        <x:v>status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="54" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>DOC-001</x:v>
+      </x:c>
+      <x:c r="B2" s="6" t="str">
+        <x:v>Repository overview</x:v>
+      </x:c>
+      <x:c r="C2" s="6" t="str">
+        <x:v>README.md</x:v>
+      </x:c>
+      <x:c r="D2" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E2" s="6" t="str">
+        <x:v>Lead systems engineer</x:v>
+      </x:c>
+      <x:c r="F2" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="54" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>DOC-002</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="str">
+        <x:v>Canonical model</x:v>
+      </x:c>
+      <x:c r="C3" s="6" t="str">
+        <x:v>00_project_control/canonical_model.json</x:v>
+      </x:c>
+      <x:c r="D3" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E3" s="6" t="str">
+        <x:v>Lead systems engineer</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="54" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>DOC-003</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>Functional design specification</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="str">
+        <x:v>13_documentation/functional_design_specification.md</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E4" s="6" t="str">
+        <x:v>Controls engineer</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>Controlled; native compile open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="54" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>DOC-004</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>Software design specification</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>13_documentation/software_design_specification.md</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>Controls engineer</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Controlled; native compile open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="54" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>DOC-005</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>PLC-NVIDIA interface control</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>02_system_architecture/interface_control_document.md</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>Controls/vision</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>Controlled; production endpoint open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>DOC-006</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>Panel design report</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>13_documentation/panel_design_report.md</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str">
+        <x:v>Electrical/panel</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>Controlled assumptions; construction open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="54" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>DOC-007</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>Electrical calculation report</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>13_documentation/electrical_calculation_report.md</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>Electrical</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>Provisional; site inputs open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="54" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>DOC-008</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>Acceptance gate status</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="str">
+        <x:v>14_qa/acceptance_gate_status.md</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="str">
+        <x:v>Independent V&amp;V</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="54" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>DOC-009</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>Engineering workbook</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>10_schedules/FC01_engineering_schedules.xlsx</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="str">
+        <x:v>Lead systems engineer</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str">
+        <x:v>Controlled generated artifact</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="54" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>DOC-010</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>Release evidence PDF</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
+        <x:v>release/FC01_release_evidence.pdf</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="str">
+        <x:v>Lead systems engineer</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="str">
+        <x:v>Controlled generated artifact</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="54" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>DOC-011</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>Release manifest</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="str">
+        <x:v>release/manifest.json</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="str">
+        <x:v>Configuration management</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>Frozen after all content</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="54" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>DOC-012</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>Native panel verification</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>09_panel_cad/revision_e/native_verification.json</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="str">
+        <x:v>Panel engineer</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="str">
+        <x:v>Native gate evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="54" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>DOC-013</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="str">
+        <x:v>Native QET verification</x:v>
+      </x:c>
+      <x:c r="C14" s="6" t="str">
+        <x:v>03_electrical/revision_e/native_verification.json</x:v>
+      </x:c>
+      <x:c r="D14" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E14" s="6" t="str">
+        <x:v>Electrical engineer</x:v>
+      </x:c>
+      <x:c r="F14" s="6" t="str">
+        <x:v>Native gate evidence when present</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="32.5" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="16.25" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="13.75" hidden="0" customWidth="1"/>
@@ -23866,7 +24222,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="18" t="str">
-        <x:v>FC01 — SIEMENS / NVIDIA ENGINEERING SCHEDULES</x:v>
+        <x:v>FC01 - SIEMENS / NVIDIA ENGINEERING SCHEDULES</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -23888,7 +24244,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="24" t="str">
-        <x:v>FICTIONAL ENGINEERING PROJECT — NOT FOR CONSTRUCTION | Revision D.1 | Professional controlled engineering-development release candidate</x:v>
+        <x:v>FICTIONAL ENGINEERING PROJECT - NOT FOR CONSTRUCTION | Revision E | Controlled native-engineering release candidate</x:v>
       </x:c>
       <x:c r="B3" s="24"/>
       <x:c r="C3" s="24"/>
@@ -23900,7 +24256,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="30" t="str">
-        <x:v>CONCEPTUAL SAFETY ARCHITECTURE — REQUIRES PROJECT-SPECIFIC RISK ASSESSMENT, DESIGN, VERIFICATION AND VALIDATION BY A QUALIFIED MACHINERY-SAFETY ENGINEER. NO PERFORMANCE LEVEL, SIL, CATEGORY, CE CONFORMITY OR REGULATORY COMPLIANCE IS CLAIMED.</x:v>
+        <x:v>CONCEPTUAL SAFETY ARCHITECTURE - REQUIRES PROJECT-SPECIFIC RISK ASSESSMENT, DESIGN, VERIFICATION AND VALIDATION BY A QUALIFIED MACHINERY-SAFETY ENGINEER. NO PERFORMANCE LEVEL, SIL, CATEGORY, CE CONFORMITY OR REGULATORY COMPLIANCE IS CLAIMED.</x:v>
       </x:c>
       <x:c r="B4" s="30"/>
       <x:c r="C4" s="30"/>
@@ -23934,7 +24290,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="D6" s="46" t="str">
-        <x:v>Native TIA/WinCC/Startdrive/PLCSIM, trained NVIDIA model, Revision-D.1 QElectroTech and Revision-D.1 panel CAD remain blocked. Historical native electrical/CAD files are byte-exact quarantined baselines. No construction, safety, native compile, FAT, SAT or model-performance claim is made.</x:v>
+        <x:v>Revision E includes source-tested poll-safe PLC/AI logic, secure asyncua integration and separately controlled native CAD/QET evidence. Native TIA/WinCC/Startdrive/PLCSIM, final site electrical design, trained NVIDIA model, target runtime, FAT/SAT, qualified safety and physical commissioning remain blocked or open exactly as listed. No construction, safety, native compile or model-performance claim is made.</x:v>
       </x:c>
       <x:c r="E6" s="46"/>
       <x:c r="F6" s="46"/>
@@ -24013,7 +24369,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="36" t="str">
-        <x:v>Controlled tests</x:v>
+        <x:v>Traceability test records</x:v>
       </x:c>
       <x:c r="B12" t="n">
         <x:f>COUNTA('Test Coverage'!A2:A100)</x:f>
@@ -24027,11 +24383,11 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="36" t="str">
-        <x:v>Open/blocked gates</x:v>
+        <x:v>PASS gates</x:v>
       </x:c>
       <x:c r="B13" t="n">
-        <x:f>COUNTIF('Acceptance Gates'!C2:C100,"BLOCKED")+COUNTIF('Acceptance Gates'!C2:C100,"OPEN")</x:f>
-        <x:v>16</x:v>
+        <x:f>COUNTIF('Acceptance Gates'!C2:C100,"PASS")</x:f>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D13" s="46"/>
       <x:c r="E13" s="46"/>
@@ -24041,18 +24397,46 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="36" t="str">
+        <x:v>PARTIAL gates</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
+        <x:f>COUNTIF('Acceptance Gates'!C2:C100,"PARTIAL")</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D14" s="46"/>
+      <x:c r="E14" s="46"/>
+      <x:c r="F14" s="46"/>
+      <x:c r="G14" s="46"/>
+      <x:c r="H14" s="46"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="36" t="str">
+        <x:v>BLOCKED + OPEN gates</x:v>
+      </x:c>
+      <x:c r="B15" t="n">
+        <x:f>COUNTIF('Acceptance Gates'!C2:C100,"BLOCKED")+COUNTIF('Acceptance Gates'!C2:C100,"OPEN")</x:f>
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D15" s="46"/>
+      <x:c r="E15" s="46"/>
+      <x:c r="F15" s="46"/>
+      <x:c r="G15" s="46"/>
+      <x:c r="H15" s="46"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="36" t="str">
         <x:v>24 VDC demand (W)</x:v>
       </x:c>
-      <x:c r="B14" t="n">
+      <x:c r="B16" t="n">
         <x:f>55+24+120+100</x:f>
         <x:v>299</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="36" t="str">
+    <x:row r="17">
+      <x:c r="A17" s="36" t="str">
         <x:v>Minimum current for 25% margin (A)</x:v>
       </x:c>
-      <x:c r="B15" t="n">
+      <x:c r="B17" t="n">
         <x:f>(55+24+120+100)/24*1.25</x:f>
         <x:v>15.572916666666668</x:v>
       </x:c>
@@ -24063,7 +24447,7 @@
     <x:mergeCell ref="A3:H3"/>
     <x:mergeCell ref="A4:H4"/>
     <x:mergeCell ref="D5:H5"/>
-    <x:mergeCell ref="D6:H13"/>
+    <x:mergeCell ref="D6:H15"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -27246,10 +27630,10 @@
         <x:v>PLC</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>One-shot request</x:v>
+        <x:v>Level-held inspection request; remains true until coherent BUSY observation or terminal result for the immutable session/inspection ID</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>OPC UA subscribed/published node</x:v>
+        <x:v>OPC UA subscribed request level; monotonic session/ID is authoritative</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
         <x:v>0</x:v>

</xml_diff>

<commit_message>
docs: record Revision E clean-clone release evidence
</commit_message>
<xml_diff>
--- a/10_schedules/FC01_engineering_schedules.xlsx
+++ b/10_schedules/FC01_engineering_schedules.xlsx
@@ -463,8 +463,8 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="DocumentRegisterTable" displayName="DocumentRegisterTable" ref="A1:F14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F14"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="DocumentRegisterTable" displayName="DocumentRegisterTable" ref="A1:F15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F15"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="document_id"/>
     <x:tableColumn id="2" name="title"/>
@@ -21695,10 +21695,10 @@
         <x:v>Manifest independently verifies</x:v>
       </x:c>
       <x:c r="C23" s="6" t="str">
-        <x:v>PARTIAL</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="D23" s="6" t="str">
-        <x:v>Pre-publication source and generated-artifact controls are implemented; final staged/HEAD manifest, upstream alignment and pushed-commit fresh-clone verification remain pending until the candidate is committed and published</x:v>
+        <x:v>Published candidate b9633c6255fe34e48a1be34afe5024935f48651e was cloned afresh from GitHub outside OneDrive and passed the complete HEAD workflow: manifest 310/310 with zero discrepancies, integrity 534/534, validator 551/551, all tests/native checks, deterministic artifacts and clean state</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -24199,6 +24199,26 @@
         <x:v>Native gate evidence when present</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="54" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>DOC-014</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="str">
+        <x:v>Post-push fresh-clone reproduction</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="str">
+        <x:v>14_qa/post_push_reproduction.md</x:v>
+      </x:c>
+      <x:c r="D15" s="6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="E15" s="6" t="str">
+        <x:v>Configuration management</x:v>
+      </x:c>
+      <x:c r="F15" s="6" t="str">
+        <x:v>Published-candidate release-integrity evidence</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
@@ -24387,7 +24407,7 @@
       </x:c>
       <x:c r="B13" t="n">
         <x:f>COUNTIF('Acceptance Gates'!C2:C100,"PASS")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D13" s="46"/>
       <x:c r="E13" s="46"/>
@@ -24401,7 +24421,7 @@
       </x:c>
       <x:c r="B14" t="n">
         <x:f>COUNTIF('Acceptance Gates'!C2:C100,"PARTIAL")</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D14" s="46"/>
       <x:c r="E14" s="46"/>

</xml_diff>

<commit_message>
fix: harden Revision F clean-clone reliability
</commit_message>
<xml_diff>
--- a/10_schedules/FC01_engineering_schedules.xlsx
+++ b/10_schedules/FC01_engineering_schedules.xlsx
@@ -27974,7 +27974,7 @@
         <x:v>TC-001..TC-032</x:v>
       </x:c>
       <x:c r="G23" s="6" t="str">
-        <x:v>32 deterministic process scenarios plus 99 source/simulator/native-contract tests, 28 deterministic vision-fault scenarios, 85 edge-service tests and 17 interface-harness tests; see the executed report</x:v>
+        <x:v>32 deterministic process scenarios plus 99 source/simulator/native-contract tests, 28 deterministic vision-fault scenarios, 86 edge-service tests and 17 interface-harness tests; see the executed report</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
@@ -28054,7 +28054,7 @@
         <x:v>Keep NVIDIA non-safety and unable to command actuators or bypass PLC interlocks</x:v>
       </x:c>
       <x:c r="C27" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D27" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28077,7 +28077,7 @@
         <x:v>Support camera, recorded-directory and explicitly synthetic non-production acquisition adapters</x:v>
       </x:c>
       <x:c r="C28" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D28" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28100,7 +28100,7 @@
         <x:v>Validate versioned configuration schema, reject unknown keys and publish configuration hashes</x:v>
       </x:c>
       <x:c r="C29" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D29" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28123,7 +28123,7 @@
         <x:v>Correlate capture acknowledgement and processing state to the immutable inspection identity</x:v>
       </x:c>
       <x:c r="C30" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D30" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28146,7 +28146,7 @@
         <x:v>Publish explicit PASS HOLD FAIL or FAULT disposition with structured reason bits</x:v>
       </x:c>
       <x:c r="C31" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D31" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28169,7 +28169,7 @@
         <x:v>Bind model, dataset and calibration identities to each accepted result</x:v>
       </x:c>
       <x:c r="C32" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D32" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28192,7 +28192,7 @@
         <x:v>Provide diagnostic UTC timestamps while retaining PLC monotonic timing as acceptance authority</x:v>
       </x:c>
       <x:c r="C33" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D33" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28215,7 +28215,7 @@
         <x:v>Expose service, camera, model, maintenance, queue and diagnostic health</x:v>
       </x:c>
       <x:c r="C34" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D34" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28238,7 +28238,7 @@
         <x:v>Fail closed when durable inspection audit records cannot be written</x:v>
       </x:c>
       <x:c r="C35" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D35" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28261,7 +28261,7 @@
         <x:v>Version and hash dataset records and split by production lot to prevent leakage</x:v>
       </x:c>
       <x:c r="C36" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D36" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28284,7 +28284,7 @@
         <x:v>Provide reproducible evaluation, FAR/FRR, threshold and latency tooling without fabricated results</x:v>
       </x:c>
       <x:c r="C37" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D37" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28307,7 +28307,7 @@
         <x:v>Define optical resolution, exposure, motion-blur, glare, focus and calibration acceptance methods</x:v>
       </x:c>
       <x:c r="C38" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D38" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28330,7 +28330,7 @@
         <x:v>Apply least-privilege certificate-based OPC UA across the controlled quality zone</x:v>
       </x:c>
       <x:c r="C39" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D39" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28353,7 +28353,7 @@
         <x:v>Retain bounded deployment rollback and independent model/configuration/calibration identities</x:v>
       </x:c>
       <x:c r="C40" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D40" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28376,7 +28376,7 @@
         <x:v>Do not retain raw production images by default and require an approved retention/privacy policy</x:v>
       </x:c>
       <x:c r="C41" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D41" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28399,7 +28399,7 @@
         <x:v>Reserve separately protected edge, camera, lighting and maintenance electrical branches</x:v>
       </x:c>
       <x:c r="C42" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D42" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28422,7 +28422,7 @@
         <x:v>Reject queue saturation, concurrent transaction reuse and results for unknown IDs</x:v>
       </x:c>
       <x:c r="C43" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D43" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28445,7 +28445,7 @@
         <x:v>Invalidate an active inspection on recipe change or unacceptable clock discontinuity</x:v>
       </x:c>
       <x:c r="C44" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D44" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28468,7 +28468,7 @@
         <x:v>Require explicit recovery and a new start following PLC or edge restart</x:v>
       </x:c>
       <x:c r="C45" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D45" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -28491,7 +28491,7 @@
         <x:v>Keep flow and level instrumentation as the primary deterministic filling measurement</x:v>
       </x:c>
       <x:c r="C46" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D46" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -31631,7 +31631,7 @@
         <x:v>Verification</x:v>
       </x:c>
       <x:c r="F19" s="6" t="str">
-        <x:v>Software-in-the-loop</x:v>
+        <x:v>Structured behavioral fault-injection model</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
@@ -31691,7 +31691,7 @@
         <x:v>Verification</x:v>
       </x:c>
       <x:c r="F22" s="6" t="str">
-        <x:v>Issued; SIL executed only</x:v>
+        <x:v>Issued; software-only behavioral fault injection executed</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -36866,7 +36866,7 @@
         <x:v>Keep NVIDIA non-safety and unable to command actuators or bypass PLC interlocks</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -36889,7 +36889,7 @@
         <x:v>Support camera, recorded-directory and explicitly synthetic non-production acquisition adapters</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -36912,7 +36912,7 @@
         <x:v>Validate versioned configuration schema, reject unknown keys and publish configuration hashes</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -36935,7 +36935,7 @@
         <x:v>Correlate capture acknowledgement and processing state to the immutable inspection identity</x:v>
       </x:c>
       <x:c r="C5" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D5" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -36958,7 +36958,7 @@
         <x:v>Publish explicit PASS HOLD FAIL or FAULT disposition with structured reason bits</x:v>
       </x:c>
       <x:c r="C6" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D6" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -36981,7 +36981,7 @@
         <x:v>Bind model, dataset and calibration identities to each accepted result</x:v>
       </x:c>
       <x:c r="C7" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D7" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37004,7 +37004,7 @@
         <x:v>Provide diagnostic UTC timestamps while retaining PLC monotonic timing as acceptance authority</x:v>
       </x:c>
       <x:c r="C8" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D8" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37027,7 +37027,7 @@
         <x:v>Expose service, camera, model, maintenance, queue and diagnostic health</x:v>
       </x:c>
       <x:c r="C9" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D9" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37050,7 +37050,7 @@
         <x:v>Fail closed when durable inspection audit records cannot be written</x:v>
       </x:c>
       <x:c r="C10" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D10" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37073,7 +37073,7 @@
         <x:v>Version and hash dataset records and split by production lot to prevent leakage</x:v>
       </x:c>
       <x:c r="C11" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D11" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37096,7 +37096,7 @@
         <x:v>Provide reproducible evaluation, FAR/FRR, threshold and latency tooling without fabricated results</x:v>
       </x:c>
       <x:c r="C12" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D12" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37119,7 +37119,7 @@
         <x:v>Define optical resolution, exposure, motion-blur, glare, focus and calibration acceptance methods</x:v>
       </x:c>
       <x:c r="C13" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D13" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37142,7 +37142,7 @@
         <x:v>Apply least-privilege certificate-based OPC UA across the controlled quality zone</x:v>
       </x:c>
       <x:c r="C14" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D14" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37165,7 +37165,7 @@
         <x:v>Retain bounded deployment rollback and independent model/configuration/calibration identities</x:v>
       </x:c>
       <x:c r="C15" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D15" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37188,7 +37188,7 @@
         <x:v>Do not retain raw production images by default and require an approved retention/privacy policy</x:v>
       </x:c>
       <x:c r="C16" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D16" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37211,7 +37211,7 @@
         <x:v>Reserve separately protected edge, camera, lighting and maintenance electrical branches</x:v>
       </x:c>
       <x:c r="C17" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D17" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37234,7 +37234,7 @@
         <x:v>Reject queue saturation, concurrent transaction reuse and results for unknown IDs</x:v>
       </x:c>
       <x:c r="C18" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D18" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37257,7 +37257,7 @@
         <x:v>Invalidate an active inspection on recipe change or unacceptable clock discontinuity</x:v>
       </x:c>
       <x:c r="C19" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D19" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37280,7 +37280,7 @@
         <x:v>Require explicit recovery and a new start following PLC or edge restart</x:v>
       </x:c>
       <x:c r="C20" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D20" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>
@@ -37303,7 +37303,7 @@
         <x:v>Keep flow and level instrumentation as the primary deterministic filling measurement</x:v>
       </x:c>
       <x:c r="C21" s="6" t="str">
-        <x:v>Review plus deterministic source/SIL tests where applicable</x:v>
+        <x:v>Review plus deterministic source tests and structured behavioral fault injection where applicable</x:v>
       </x:c>
       <x:c r="D21" s="6" t="str">
         <x:v>Implemented locally where possible; external native/data/hardware acceptance remains explicit</x:v>

</xml_diff>

<commit_message>
chore: attest Revision F clean-clone release
</commit_message>
<xml_diff>
--- a/10_schedules/FC01_engineering_schedules.xlsx
+++ b/10_schedules/FC01_engineering_schedules.xlsx
@@ -31228,10 +31228,10 @@
         <x:v>Manifest independently verifies</x:v>
       </x:c>
       <x:c r="C23" s="6" t="str">
-        <x:v>PARTIAL</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="D23" s="6" t="str">
-        <x:v>Manifest and clean-clone release-integrity gate closes only after the final Revision-F commit is pushed and reproduced</x:v>
+        <x:v>Published candidate f6e9f3b1e928a2e04d21913caac2547469b0f647 reproduced from GitHub with 425/425 manifest entries, zero discrepancies and final Git-clean assertion</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -32082,7 +32082,7 @@
       </x:c>
       <x:c r="B13" t="n">
         <x:f>COUNTIF('Acceptance Gates'!C2:C100,"PASS")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D13" s="46"/>
       <x:c r="E13" s="46"/>
@@ -32096,7 +32096,7 @@
       </x:c>
       <x:c r="B14" t="n">
         <x:f>COUNTIF('Acceptance Gates'!C2:C100,"PARTIAL")</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D14" s="46"/>
       <x:c r="E14" s="46"/>

</xml_diff>

<commit_message>
feat: establish Revision G native cloud execution package
</commit_message>
<xml_diff>
--- a/10_schedules/FC01_engineering_schedules.xlsx
+++ b/10_schedules/FC01_engineering_schedules.xlsx
@@ -14,20 +14,21 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NVIDIA Electrical" sheetId="10" r:id="rId13"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NVIDIA Versions" sheetId="11" r:id="rId14"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revision-F Gaps" sheetId="12" r:id="rId15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network Nodes" sheetId="13" r:id="rId16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terminal Plan" sheetId="14" r:id="rId17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Point-to-Point" sheetId="15" r:id="rId18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cable Schedule" sheetId="16" r:id="rId19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wire List" sheetId="17" r:id="rId20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="18" r:id="rId21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Load Budget" sheetId="19" r:id="rId22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Placement" sheetId="20" r:id="rId23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements Trace" sheetId="21" r:id="rId24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Coverage" sheetId="22" r:id="rId25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input Requests" sheetId="23" r:id="rId26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Gates" sheetId="24" r:id="rId27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document Register" sheetId="25" r:id="rId28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Summary" sheetId="26" r:id="rId29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revision-G Gates" sheetId="13" r:id="rId16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network Nodes" sheetId="14" r:id="rId17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terminal Plan" sheetId="15" r:id="rId18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Point-to-Point" sheetId="16" r:id="rId19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cable Schedule" sheetId="17" r:id="rId20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wire List" sheetId="18" r:id="rId21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="19" r:id="rId22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Load Budget" sheetId="20" r:id="rId23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Placement" sheetId="21" r:id="rId24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements Trace" sheetId="22" r:id="rId25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Coverage" sheetId="23" r:id="rId26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input Requests" sheetId="24" r:id="rId27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Gates" sheetId="25" r:id="rId28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document Register" sheetId="26" r:id="rId29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Summary" sheetId="27" r:id="rId30"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -300,7 +301,26 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="NetworkNodesTable" displayName="NetworkNodesTable" ref="A1:H8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="RevisionGGatesTable" displayName="RevisionGGatesTable" ref="A1:J15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J15"/>
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="gate_id"/>
+    <x:tableColumn id="2" name="requirement"/>
+    <x:tableColumn id="3" name="current_evidence"/>
+    <x:tableColumn id="4" name="current_status"/>
+    <x:tableColumn id="5" name="missing_input"/>
+    <x:tableColumn id="6" name="responsible_agent"/>
+    <x:tableColumn id="7" name="planned_action"/>
+    <x:tableColumn id="8" name="acceptance_evidence"/>
+    <x:tableColumn id="9" name="external_dependency"/>
+    <x:tableColumn id="10" name="final_disposition"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="NetworkNodesTable" displayName="NetworkNodesTable" ref="A1:H8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:H8"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="node"/>
@@ -316,8 +336,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="TerminalPlanTable" displayName="TerminalPlanTable" ref="A1:Q85" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="TerminalPlanTable" displayName="TerminalPlanTable" ref="A1:Q85" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:Q85"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="terminal"/>
@@ -342,8 +362,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="PointtoPointTable" displayName="PointtoPointTable" ref="A1:V119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="PointtoPointTable" displayName="PointtoPointTable" ref="A1:V119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:V119"/>
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="signal"/>
@@ -373,8 +393,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="CableScheduleTable" displayName="CableScheduleTable" ref="A1:L23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="CableScheduleTable" displayName="CableScheduleTable" ref="A1:L23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:L23"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="cable_id"/>
@@ -394,8 +414,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="WireListTable" displayName="WireListTable" ref="A1:V119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="WireListTable" displayName="WireListTable" ref="A1:V119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:V119"/>
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="signal"/>
@@ -425,8 +445,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="BOMTable" displayName="BOMTable" ref="A1:J63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="BOMTable" displayName="BOMTable" ref="A1:J63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:J63"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="item"/>
@@ -439,21 +459,6 @@
     <x:tableColumn id="8" name="scope"/>
     <x:tableColumn id="9" name="basis_or_blocker"/>
     <x:tableColumn id="10" name="full_designation"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="LoadBudgetTable" displayName="LoadBudgetTable" ref="A1:F11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F11"/>
-  <x:tableColumns count="6">
-    <x:tableColumn id="1" name="load"/>
-    <x:tableColumn id="2" name="voltage"/>
-    <x:tableColumn id="3" name="nominal_w"/>
-    <x:tableColumn id="4" name="demand_factor"/>
-    <x:tableColumn id="5" name="demand_w"/>
-    <x:tableColumn id="6" name="basis"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -478,7 +483,22 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="PanelPlacementTable" displayName="PanelPlacementTable" ref="A1:P15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="LoadBudgetTable" displayName="LoadBudgetTable" ref="A1:F11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F11"/>
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="load"/>
+    <x:tableColumn id="2" name="voltage"/>
+    <x:tableColumn id="3" name="nominal_w"/>
+    <x:tableColumn id="4" name="demand_factor"/>
+    <x:tableColumn id="5" name="demand_w"/>
+    <x:tableColumn id="6" name="basis"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="PanelPlacementTable" displayName="PanelPlacementTable" ref="A1:P15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:P15"/>
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="tag"/>
@@ -502,8 +522,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="RequirementsTraceTable" displayName="RequirementsTraceTable" ref="A1:G46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="RequirementsTraceTable" displayName="RequirementsTraceTable" ref="A1:G46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:G46"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="requirement_id"/>
@@ -518,8 +538,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="TestCoverageTable" displayName="TestCoverageTable" ref="A1:G73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="TestCoverageTable" displayName="TestCoverageTable" ref="A1:G73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:G73"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="test_id"/>
@@ -534,8 +554,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="InputRequestsTable" displayName="InputRequestsTable" ref="A1:G29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="InputRequestsTable" displayName="InputRequestsTable" ref="A1:G29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:G29"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="request_id"/>
@@ -550,8 +570,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="AcceptanceGatesTable" displayName="AcceptanceGatesTable" ref="A1:D23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="AcceptanceGatesTable" displayName="AcceptanceGatesTable" ref="A1:D23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:D23"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="gate"/>
@@ -563,9 +583,9 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="DocumentRegisterTable" displayName="DocumentRegisterTable" ref="A1:F32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F32"/>
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="DocumentRegisterTable" displayName="DocumentRegisterTable" ref="A1:F46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F46"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="document_id"/>
     <x:tableColumn id="2" name="title"/>
@@ -2579,6 +2599,510 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="10.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="33.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="33.75" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="33.75" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="19.3799991607666" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="31.5" customHeight="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>gate_id</x:v>
+      </x:c>
+      <x:c r="B1" s="12" t="str">
+        <x:v>requirement</x:v>
+      </x:c>
+      <x:c r="C1" s="12" t="str">
+        <x:v>current_evidence</x:v>
+      </x:c>
+      <x:c r="D1" s="12" t="str">
+        <x:v>current_status</x:v>
+      </x:c>
+      <x:c r="E1" s="12" t="str">
+        <x:v>missing_input</x:v>
+      </x:c>
+      <x:c r="F1" s="12" t="str">
+        <x:v>responsible_agent</x:v>
+      </x:c>
+      <x:c r="G1" s="12" t="str">
+        <x:v>planned_action</x:v>
+      </x:c>
+      <x:c r="H1" s="12" t="str">
+        <x:v>acceptance_evidence</x:v>
+      </x:c>
+      <x:c r="I1" s="12" t="str">
+        <x:v>external_dependency</x:v>
+      </x:c>
+      <x:c r="J1" s="12" t="str">
+        <x:v>final_disposition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="54" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>G0-01</x:v>
+      </x:c>
+      <x:c r="B2" s="6" t="str">
+        <x:v>Reviewable two-environment Google Cloud architecture</x:v>
+      </x:c>
+      <x:c r="C2" s="6" t="str">
+        <x:v>cloud/architecture.md and cloud/terraform</x:v>
+      </x:c>
+      <x:c r="D2" s="6" t="str">
+        <x:v>VERIFIED</x:v>
+      </x:c>
+      <x:c r="E2" s="6" t="str">
+        <x:v>None for design</x:v>
+      </x:c>
+      <x:c r="F2" s="6" t="str">
+        <x:v>Cloud/DevSecOps workstream</x:v>
+      </x:c>
+      <x:c r="G2" s="6" t="str">
+        <x:v>Retain architecture under release control</x:v>
+      </x:c>
+      <x:c r="H2" s="6" t="str">
+        <x:v>Revision-G static security verification</x:v>
+      </x:c>
+      <x:c r="I2" s="6" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="J2" s="6" t="str">
+        <x:v>VERIFIED - design only; no resources created</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="54" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>G0-02</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="str">
+        <x:v>Terraform format, native validate and non-destructive plan</x:v>
+      </x:c>
+      <x:c r="C3" s="6" t="str">
+        <x:v>Static HCL/security checks pass; Terraform CLI absent</x:v>
+      </x:c>
+      <x:c r="D3" s="6" t="str">
+        <x:v>BLOCKED BY EXTERNAL SYSTEM</x:v>
+      </x:c>
+      <x:c r="E3" s="6" t="str">
+        <x:v>Approved Terraform/OpenTofu CLI, Google project, billing identity and ADC</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="str">
+        <x:v>Cloud owner</x:v>
+      </x:c>
+      <x:c r="G3" s="6" t="str">
+        <x:v>Run cloud/scripts/plan_cloud.ps1 after consolidated approval</x:v>
+      </x:c>
+      <x:c r="H3" s="6" t="str">
+        <x:v>fmt/validate/plan logs and plan SHA-256</x:v>
+      </x:c>
+      <x:c r="I3" s="6" t="str">
+        <x:v>User cloud authorization and tool approval</x:v>
+      </x:c>
+      <x:c r="J3" s="6" t="str">
+        <x:v>BLOCKED - no plan or apply claimed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="54" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>G0-03</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>Cloud security, budget and shutdown controls</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="str">
+        <x:v>No external IPs, IAP-only ingress, separate service accounts, budgets, schedules and bucket controls encoded</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="str">
+        <x:v>IMPLEMENTABLE NOW</x:v>
+      </x:c>
+      <x:c r="E4" s="6" t="str">
+        <x:v>Project-specific IAM principals, billing account and reviewed budget</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>Cloud security owner</x:v>
+      </x:c>
+      <x:c r="G4" s="6" t="str">
+        <x:v>Parameterize and plan only after approval</x:v>
+      </x:c>
+      <x:c r="H4" s="6" t="str">
+        <x:v>Reviewed plan plus Security Command Center/IAM evidence after apply</x:v>
+      </x:c>
+      <x:c r="I4" s="6" t="str">
+        <x:v>Cloud project and billing access</x:v>
+      </x:c>
+      <x:c r="J4" s="6" t="str">
+        <x:v>DEPLOYABLE; NOT PROVISIONED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="54" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>G1-01</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>Authorized TIA Portal V20 native project and reopen</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>Portal executable 2000.0.9501.1 and Openness V20 assemblies installed; no genuine AP20</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>REQUIRES LICENCE</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>Valid STEP 7/WinCC licences and Siemens TIA Openness group membership</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Licensed Siemens engineer</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>Execute siemens_native handoff and import controlled sources</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str">
+        <x:v>Native AP20/ZAP20, reopen log and hashes</x:v>
+      </x:c>
+      <x:c r="I5" s="6" t="str">
+        <x:v>Licence, authorization and qualified operator</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
+        <x:v>BLOCKED - no AP20/ZAP20 fabricated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="54" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>G1-02</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>Native PLC, hardware and HMI compile</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>99 source/simulator contract tests; import-ready SCL/HMI tables</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>REQUIRES LICENCE</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>Authorized TIA session and catalog confirmation</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>Licensed Siemens engineer</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>Compile and disposition every warning</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="str">
+        <x:v>Raw native compile logs and screenshots</x:v>
+      </x:c>
+      <x:c r="I6" s="6" t="str">
+        <x:v>TIA licence/authorization</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="str">
+        <x:v>BLOCKED - source tests are not native compilation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>G1-03</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>Startdrive and PLCSIM execution</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>Neither Startdrive nor PLCSIM is installed</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>REQUIRES LICENCE</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str">
+        <x:v>Approved installers/licences plus motor and pump data</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>Drives/controls owner</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str">
+        <x:v>Install through approved Siemens channel, configure, compile and simulate</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="str">
+        <x:v>Product inventory, native compile and PLCSIM traces</x:v>
+      </x:c>
+      <x:c r="I7" s="6" t="str">
+        <x:v>Software, licences and machine data</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="str">
+        <x:v>BLOCKED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="54" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>G2-01</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>Production-shaped fail-closed PLC-AI edge contract</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>47-node contract, encrypted asyncua integration and immutable ACK behavior; 86 edge and 17 harness tests</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>VERIFIED</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>Production S7/Jetson endpoint for deployment acceptance</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>NVIDIA/controls owners</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="str">
+        <x:v>Retain software contract and repeat on target</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="str">
+        <x:v>Automated unit/integration/fault evidence</x:v>
+      </x:c>
+      <x:c r="I8" s="6" t="str">
+        <x:v>Target endpoint for production validation</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="str">
+        <x:v>VERIFIED AS SOFTWARE-ONLY NON-SAFETY CONTRACT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="54" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>G2-02</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>Dataset provenance, taxonomy and split controls</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="str">
+        <x:v>Acquisition/labeling plans, empty controlled manifest and executable validation/split tooling</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>REQUIRES REAL DATA</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="str">
+        <x:v>Approved representative multi-lot images and annotations</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="str">
+        <x:v>Vision product owner</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="str">
+        <x:v>Collect and double-review approved real data</x:v>
+      </x:c>
+      <x:c r="H9" s="6" t="str">
+        <x:v>Hashed manifest, provenance, class balance, leakage/duplicate review</x:v>
+      </x:c>
+      <x:c r="I9" s="6" t="str">
+        <x:v>Real process samples, camera/lighting and data approval</x:v>
+      </x:c>
+      <x:c r="J9" s="6" t="str">
+        <x:v>PIPELINE READY; DATASET ABSENT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="54" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>G2-03</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>Real TAO training, independent evaluation and deployment artifacts</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>Pinned configuration templates and synthetic fail-closed smoke only</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>REQUIRES REAL DATA</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="str">
+        <x:v>Approved dataset, Linux GPU runtime and selected architecture</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str">
+        <x:v>Vision/MLOps owner</x:v>
+      </x:c>
+      <x:c r="G10" s="6" t="str">
+        <x:v>Train, evaluate, export ONNX and generate target TensorRT engine</x:v>
+      </x:c>
+      <x:c r="H10" s="6" t="str">
+        <x:v>Raw logs, held-out metrics, model card, artifact hashes and target latency</x:v>
+      </x:c>
+      <x:c r="I10" s="6" t="str">
+        <x:v>Dataset, GPU environment and model approval</x:v>
+      </x:c>
+      <x:c r="J10" s="6" t="str">
+        <x:v>BLOCKED - no model or metric claimed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="54" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>G2-04</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>DeepStream/TAO/TensorRT native runtime</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
+        <x:v>RTX 5060 driver 595.95 is present; nvcc, Docker, TAO, TensorRT and DeepStream absent</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>REQUIRES USER APPROVAL</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="str">
+        <x:v>Approved Ubuntu 24.04/container runtime installation or cloud GPU plan</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="str">
+        <x:v>NVIDIA platform owner</x:v>
+      </x:c>
+      <x:c r="G11" s="6" t="str">
+        <x:v>Execute pinned environment runbook after approval</x:v>
+      </x:c>
+      <x:c r="H11" s="6" t="str">
+        <x:v>Native version logs, container digest, SBOM and measured smoke/latency logs</x:v>
+      </x:c>
+      <x:c r="I11" s="6" t="str">
+        <x:v>Installation approval, registry terms and runtime</x:v>
+      </x:c>
+      <x:c r="J11" s="6" t="str">
+        <x:v>BLOCKED - GPU inventory only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="54" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>G3A-01</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>Controlled commissioning procedures and blank records</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="str">
+        <x:v>commissioning directory contains FAT/SAT, inspection, calibration, I/O and safety-review templates</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>VERIFIED</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="str">
+        <x:v>None for controlled blank templates</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>Commissioning preparation owner</x:v>
+      </x:c>
+      <x:c r="G12" s="6" t="str">
+        <x:v>Issue to qualified execution team</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="str">
+        <x:v>Revision-G consistency and schema verification</x:v>
+      </x:c>
+      <x:c r="I12" s="6" t="str">
+        <x:v>None for preparation</x:v>
+      </x:c>
+      <x:c r="J12" s="6" t="str">
+        <x:v>VERIFIED AS DOCUMENTATION ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="54" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>G3A-02</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>Construction information reconciled to final site/equipment inputs</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>Deterministic fictional schedules exist; Revision-F vision electrical delta and site calculations remain provisional</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="str">
+        <x:v>REQUIRES REAL DATA</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="str">
+        <x:v>Supply, earthing, fault current, motors, routes, ambient, enclosure and selected vision hardware</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="str">
+        <x:v>Qualified electrical designer</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="str">
+        <x:v>Finalize calculations and apply controlled QET/CAD change</x:v>
+      </x:c>
+      <x:c r="H13" s="6" t="str">
+        <x:v>Approved calculations, updated native QET/CAD and construction review</x:v>
+      </x:c>
+      <x:c r="I13" s="6" t="str">
+        <x:v>Site/equipment data and qualified review</x:v>
+      </x:c>
+      <x:c r="J13" s="6" t="str">
+        <x:v>PARTIAL - not construction ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="54" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>G3B-01</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="str">
+        <x:v>Physical FAT/SAT and commissioning evidence</x:v>
+      </x:c>
+      <x:c r="C14" s="6" t="str">
+        <x:v>Blank records only</x:v>
+      </x:c>
+      <x:c r="D14" s="6" t="str">
+        <x:v>REQUIRES HARDWARE</x:v>
+      </x:c>
+      <x:c r="E14" s="6" t="str">
+        <x:v>Built panel/machine, calibrated instruments, site and qualified testers</x:v>
+      </x:c>
+      <x:c r="F14" s="6" t="str">
+        <x:v>Commissioning manager</x:v>
+      </x:c>
+      <x:c r="G14" s="6" t="str">
+        <x:v>Execute controlled procedures without prefilled values</x:v>
+      </x:c>
+      <x:c r="H14" s="6" t="str">
+        <x:v>Signed raw measurements, punch closure and as-built redlines</x:v>
+      </x:c>
+      <x:c r="I14" s="6" t="str">
+        <x:v>Hardware and personnel</x:v>
+      </x:c>
+      <x:c r="J14" s="6" t="str">
+        <x:v>0% EXECUTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="54" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>G3C-01</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="str">
+        <x:v>Qualified electrical and machinery-safety review</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="str">
+        <x:v>Conceptual boundary, hazard assumptions and validation template only</x:v>
+      </x:c>
+      <x:c r="D15" s="6" t="str">
+        <x:v>REQUIRES QUALIFIED PERSON</x:v>
+      </x:c>
+      <x:c r="E15" s="6" t="str">
+        <x:v>Named competent electrical and machinery-safety engineers plus project risk assessment</x:v>
+      </x:c>
+      <x:c r="F15" s="6" t="str">
+        <x:v>Project owner</x:v>
+      </x:c>
+      <x:c r="G15" s="6" t="str">
+        <x:v>Submit qualified-review handoff</x:v>
+      </x:c>
+      <x:c r="H15" s="6" t="str">
+        <x:v>Signed review, validated calculations and safety lifecycle records</x:v>
+      </x:c>
+      <x:c r="I15" s="6" t="str">
+        <x:v>Qualified people and organization approval</x:v>
+      </x:c>
+      <x:c r="J15" s="6" t="str">
+        <x:v>0% EXECUTED</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="19.3799991607666" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="19.3799991607666" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="19.3799991607666" hidden="0" customWidth="1"/>
@@ -2805,7 +3329,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -7155,7 +7679,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -14313,7 +14837,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -15213,7 +15737,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -22371,7 +22895,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -24207,246 +24731,6 @@
       </x:c>
       <x:c r="J63" s="6" t="str">
         <x:v>=FC01+FLD-B131</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="19.3799991607666" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="19.3799991607666" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="19.3799991607666" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="19.3799991607666" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="19.3799991607666" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="33.75" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="31.5" customHeight="1">
-      <x:c r="A1" s="12" t="str">
-        <x:v>load</x:v>
-      </x:c>
-      <x:c r="B1" s="12" t="str">
-        <x:v>voltage</x:v>
-      </x:c>
-      <x:c r="C1" s="12" t="str">
-        <x:v>nominal_w</x:v>
-      </x:c>
-      <x:c r="D1" s="12" t="str">
-        <x:v>demand_factor</x:v>
-      </x:c>
-      <x:c r="E1" s="12" t="str">
-        <x:v>demand_w</x:v>
-      </x:c>
-      <x:c r="F1" s="12" t="str">
-        <x:v>basis</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="54" customHeight="1">
-      <x:c r="A2" s="6" t="str">
-        <x:v>PLC CPU and I/O</x:v>
-      </x:c>
-      <x:c r="B2" s="6" t="str">
-        <x:v>24 VDC</x:v>
-      </x:c>
-      <x:c r="C2" s="6" t="str">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="D2" s="6" t="str">
-        <x:v>1.0</x:v>
-      </x:c>
-      <x:c r="E2" s="6" t="str">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="F2" s="6" t="str">
-        <x:v>Preliminary allowance; verify Siemens configuration</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="54" customHeight="1">
-      <x:c r="A3" s="6" t="str">
-        <x:v>HMI</x:v>
-      </x:c>
-      <x:c r="B3" s="6" t="str">
-        <x:v>24 VDC</x:v>
-      </x:c>
-      <x:c r="C3" s="6" t="str">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D3" s="6" t="str">
-        <x:v>1.0</x:v>
-      </x:c>
-      <x:c r="E3" s="6" t="str">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="F3" s="6" t="str">
-        <x:v>Maximum-current allowance from product data</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="54" customHeight="1">
-      <x:c r="A4" s="6" t="str">
-        <x:v>Relays, sensors and solenoids</x:v>
-      </x:c>
-      <x:c r="B4" s="6" t="str">
-        <x:v>24 VDC</x:v>
-      </x:c>
-      <x:c r="C4" s="6" t="str">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="D4" s="6" t="str">
-        <x:v>0.8</x:v>
-      </x:c>
-      <x:c r="E4" s="6" t="str">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="F4" s="6" t="str">
-        <x:v>Duty-cycle allowance; inrush not finalized</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="54" customHeight="1">
-      <x:c r="A5" s="6" t="str">
-        <x:v>Vision edge compute allowance</x:v>
-      </x:c>
-      <x:c r="B5" s="6" t="str">
-        <x:v>24 VDC</x:v>
-      </x:c>
-      <x:c r="C5" s="6" t="str">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="str">
-        <x:v>1.0</x:v>
-      </x:c>
-      <x:c r="E5" s="6" t="str">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="F5" s="6" t="str">
-        <x:v>Provisional branch -F220; carrier/input/inrush unconfirmed</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="54" customHeight="1">
-      <x:c r="A6" s="6" t="str">
-        <x:v>Vision camera allowance</x:v>
-      </x:c>
-      <x:c r="B6" s="6" t="str">
-        <x:v>24 VDC</x:v>
-      </x:c>
-      <x:c r="C6" s="6" t="str">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="D6" s="6" t="str">
-        <x:v>1.0</x:v>
-      </x:c>
-      <x:c r="E6" s="6" t="str">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="F6" s="6" t="str">
-        <x:v>Provisional branch -F221; PoE not assumed</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="54" customHeight="1">
-      <x:c r="A7" s="6" t="str">
-        <x:v>Vision lighting allowance</x:v>
-      </x:c>
-      <x:c r="B7" s="6" t="str">
-        <x:v>24 VDC</x:v>
-      </x:c>
-      <x:c r="C7" s="6" t="str">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="str">
-        <x:v>1.0</x:v>
-      </x:c>
-      <x:c r="E7" s="6" t="str">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F7" s="6" t="str">
-        <x:v>Provisional branch -F222; pulse duty/inrush unconfirmed</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="54" customHeight="1">
-      <x:c r="A8" s="6" t="str">
-        <x:v>Vision service/network allowance</x:v>
-      </x:c>
-      <x:c r="B8" s="6" t="str">
-        <x:v>24 VDC</x:v>
-      </x:c>
-      <x:c r="C8" s="6" t="str">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D8" s="6" t="str">
-        <x:v>1.0</x:v>
-      </x:c>
-      <x:c r="E8" s="6" t="str">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="F8" s="6" t="str">
-        <x:v>Provisional branch -F223; maintenance-only service</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="54" customHeight="1">
-      <x:c r="A9" s="6" t="str">
-        <x:v>24 VDC subtotal</x:v>
-      </x:c>
-      <x:c r="B9" s="6" t="str">
-        <x:v>24 VDC</x:v>
-      </x:c>
-      <x:c r="C9" s="6" t="str">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="D9" s="6" t="str">
-        <x:v>N/A</x:v>
-      </x:c>
-      <x:c r="E9" s="6" t="str">
-        <x:v>299</x:v>
-      </x:c>
-      <x:c r="F9" s="6" t="str">
-        <x:v>12.458 A demand; 20 A concept leaves 7.542 A (37.71% of rating) unused; minimum 15.573 A for 25% demand margin before inrush/derating</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="54" customHeight="1">
-      <x:c r="A10" s="6" t="str">
-        <x:v>Conveyor drive</x:v>
-      </x:c>
-      <x:c r="B10" s="6" t="str">
-        <x:v>400 VAC</x:v>
-      </x:c>
-      <x:c r="C10" s="6" t="str">
-        <x:v>750</x:v>
-      </x:c>
-      <x:c r="D10" s="6" t="str">
-        <x:v>1.0</x:v>
-      </x:c>
-      <x:c r="E10" s="6" t="str">
-        <x:v>750</x:v>
-      </x:c>
-      <x:c r="F10" s="6" t="str">
-        <x:v>Motor nameplate not supplied</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="54" customHeight="1">
-      <x:c r="A11" s="6" t="str">
-        <x:v>Pump drive</x:v>
-      </x:c>
-      <x:c r="B11" s="6" t="str">
-        <x:v>400 VAC</x:v>
-      </x:c>
-      <x:c r="C11" s="6" t="str">
-        <x:v>750</x:v>
-      </x:c>
-      <x:c r="D11" s="6" t="str">
-        <x:v>1.0</x:v>
-      </x:c>
-      <x:c r="E11" s="6" t="str">
-        <x:v>750</x:v>
-      </x:c>
-      <x:c r="F11" s="6" t="str">
-        <x:v>Pump curve/motor nameplate not supplied</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -26662,6 +26946,246 @@
     <x:col min="1" max="1" width="19.3799991607666" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="19.3799991607666" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="33.75" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="31.5" customHeight="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>load</x:v>
+      </x:c>
+      <x:c r="B1" s="12" t="str">
+        <x:v>voltage</x:v>
+      </x:c>
+      <x:c r="C1" s="12" t="str">
+        <x:v>nominal_w</x:v>
+      </x:c>
+      <x:c r="D1" s="12" t="str">
+        <x:v>demand_factor</x:v>
+      </x:c>
+      <x:c r="E1" s="12" t="str">
+        <x:v>demand_w</x:v>
+      </x:c>
+      <x:c r="F1" s="12" t="str">
+        <x:v>basis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="54" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>PLC CPU and I/O</x:v>
+      </x:c>
+      <x:c r="B2" s="6" t="str">
+        <x:v>24 VDC</x:v>
+      </x:c>
+      <x:c r="C2" s="6" t="str">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D2" s="6" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E2" s="6" t="str">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F2" s="6" t="str">
+        <x:v>Preliminary allowance; verify Siemens configuration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="54" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>HMI</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="str">
+        <x:v>24 VDC</x:v>
+      </x:c>
+      <x:c r="C3" s="6" t="str">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="D3" s="6" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E3" s="6" t="str">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="str">
+        <x:v>Maximum-current allowance from product data</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="54" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>Relays, sensors and solenoids</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>24 VDC</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="str">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="str">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="E4" s="6" t="str">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>Duty-cycle allowance; inrush not finalized</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="54" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>Vision edge compute allowance</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>24 VDC</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Provisional branch -F220; carrier/input/inrush unconfirmed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="54" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>Vision camera allowance</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>24 VDC</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>Provisional branch -F221; PoE not assumed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>Vision lighting allowance</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>24 VDC</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>Provisional branch -F222; pulse duty/inrush unconfirmed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="54" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>Vision service/network allowance</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>24 VDC</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>Provisional branch -F223; maintenance-only service</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="54" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>24 VDC subtotal</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>24 VDC</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="str">
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="str">
+        <x:v>299</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="str">
+        <x:v>12.458 A demand; 20 A concept leaves 7.542 A (37.71% of rating) unused; minimum 15.573 A for 25% demand margin before inrush/derating</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="54" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>Conveyor drive</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>400 VAC</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="str">
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str">
+        <x:v>Motor nameplate not supplied</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="54" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>Pump drive</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>400 VAC</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="str">
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="str">
+        <x:v>Pump curve/motor nameplate not supplied</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="19.3799991607666" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="19.3799991607666" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="19.3799991607666" hidden="0" customWidth="1"/>
@@ -27435,7 +27959,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -28514,7 +29038,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -30214,7 +30738,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -30902,7 +31426,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -30937,7 +31461,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
-        <x:v>Revision-F requirements and evidence are traceable; identified owner approval remains absent</x:v>
+        <x:v>Revision-G requirements, execution gates and evidence are traceable; owner and qualified-human approvals remain absent</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="54" customHeight="1">
@@ -30951,7 +31475,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Core canonical/interface schedules reconcile; the standalone Revision-F NVIDIA electrical delta is internally consistent but is not yet incorporated into canonical BOM/terminal/cable/P2P/QET/CAD authorities</x:v>
+        <x:v>Core authorities reconcile; the Revision-F NVIDIA electrical delta remains provisional and outside final QET/CAD/construction authorities</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="54" customHeight="1">
@@ -30965,7 +31489,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>V20/FW4.0 source baseline and selected envelopes documented; authorized native catalog confirmation and delivered-state evidence remain open</x:v>
+        <x:v>TIA V20/Openness installation is inventoried exactly; authorized native catalog confirmation and delivered hardware remain open</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="54" customHeight="1">
@@ -30979,7 +31503,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D5" s="6" t="str">
-        <x:v>No genuine AP20 project; active identity is not TIA Engineer/Openness-authorized and V20 entitlement is unproven</x:v>
+        <x:v>TIA V20 exists but no licensed/Openness-authorized session or genuine AP20 project was available</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
@@ -30993,7 +31517,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D6" s="6" t="str">
-        <x:v>No genuine ZAP20 archive exists; native authorized project creation/restoration was not available</x:v>
+        <x:v>No genuine ZAP20 archive exists; no native archive was fabricated</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -31007,7 +31531,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D7" s="6" t="str">
-        <x:v>Expanded import-ready SCL/source contracts pass locally; native TIA V20 compile was not run</x:v>
+        <x:v>99 Siemens/source/simulator contract tests pass; native TIA compile was not run</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
@@ -31021,7 +31545,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D8" s="6" t="str">
-        <x:v>Expanded HMI definitions are source-controlled; native WinCC Unified compile/usability review was not run</x:v>
+        <x:v>HMI definitions are controlled; native WinCC Unified compile/usability review was not run</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
@@ -31035,7 +31559,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D9" s="6" t="str">
-        <x:v>Startdrive is not installed; motor, pump and site inputs are also missing</x:v>
+        <x:v>Startdrive is absent and motor/pump/site data remain unconfirmed</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -31049,7 +31573,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D10" s="6" t="str">
-        <x:v>PLCSIM/PLCSIM Advanced are not installed; deterministic Python evidence is explicitly independent</x:v>
+        <x:v>PLCSIM/PLCSIM Advanced are absent; Python evidence is independent and explicitly non-native</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -31063,7 +31587,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D11" s="6" t="str">
-        <x:v>Exact controlled Revision-E QET hash reopened natively with 26/26 folios; automatic cross-reference resolution remains unsupported</x:v>
+        <x:v>Inherited exact-hash 26-folio QET reopen remains valid; executable was not found for a new Revision-G execution and automatic cross-references remain unsupported</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -31077,7 +31601,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D12" s="6" t="str">
-        <x:v>Native 26-page PDF export completed; all pages were reviewed, with one clipped in-body statement on folio 25 and dense text noted</x:v>
+        <x:v>Inherited 26-page native export was reviewed; folio 25 clipping/density limitation remains open</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
@@ -31091,7 +31615,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D13" s="6" t="str">
-        <x:v>FreeCADCmd independently reopened 165 objects / 148 controlled solids; STEP retained 148 solids; IGES retained bounded face geometry; DXF entities and 30 scheduled holes reconciled</x:v>
+        <x:v>FreeCADCmd 1.1.3 re-executed in Revision G: 165 objects, 148 solids, zero invalid shapes</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="54" customHeight="1">
@@ -31105,7 +31629,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D14" s="6" t="str">
-        <x:v>FreeCADCmd independently reopened 165 objects / 148 controlled solids; STEP retained 148 solids; IGES retained bounded face geometry; DXF entities and 30 scheduled holes reconciled</x:v>
+        <x:v>Revision-G FreeCAD execution reimported STEP/IGES/DXF and reconciled 30 mounting holes</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
@@ -31119,7 +31643,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D15" s="6" t="str">
-        <x:v>Revision-E panel CAD remains natively verified; Revision-F electrical delta uses provisional carrier/camera/light envelopes and is not incorporated into QET/CAD</x:v>
+        <x:v>Revision-E CAD remains natively verified; final selected vision envelopes and electrical delta incorporation remain open</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
@@ -31133,7 +31657,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D16" s="6" t="str">
-        <x:v>Supply, earthing, fault current, motors/pump, cable routes, installation method, ambient and enclosure/site requirements remain unconfirmed</x:v>
+        <x:v>Supply, earthing, fault current, motor/pump, routes, installation, ambient and enclosure inputs remain absent</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
@@ -31147,7 +31671,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D17" s="6" t="str">
-        <x:v>Dataset tooling, schema, collection matrix and leakage-safe split checks are ready; no representative labeled dataset exists</x:v>
+        <x:v>Dataset acquisition/labeling/schema tooling is controlled; representative real data is absent</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
@@ -31161,7 +31685,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D18" s="6" t="str">
-        <x:v>Training/evaluation tooling is ready; no approved dataset, training run, model or defensible production metrics exist</x:v>
+        <x:v>Training/evaluation configuration is ready; no approved dataset, training run, model or metric exists</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
@@ -31175,7 +31699,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D19" s="6" t="str">
-        <x:v>DeepStream 9.1/TAO 7.0.1 policy is documented; CUDA/TAO/TensorRT/DeepStream/Docker and target hardware are absent</x:v>
+        <x:v>RTX 5060 driver query passed; CUDA, Docker, TAO, TensorRT, DeepStream and target Jetson/cloud runtime are absent</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
@@ -31189,7 +31713,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D20" s="6" t="str">
-        <x:v>Source, edge, durable-audit, encrypted OPC UA and interface tests pass locally; native SCL enum binding, production S7/Jetson endpoint and physical timing remain unverified</x:v>
+        <x:v>Fail-closed edge/OPC UA/harness/synthetic-authorization tests pass; production S7/Jetson endpoint and physical timing remain unverified</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
@@ -31203,7 +31727,7 @@
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="D21" s="6" t="str">
-        <x:v>Controlled procedures issued; no FAT, SAT or commissioning was executed</x:v>
+        <x:v>G3A procedures and blank records are issued; no FAT, SAT or commissioning measurement was executed</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="54" customHeight="1">
@@ -31217,7 +31741,7 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D22" s="6" t="str">
-        <x:v>Project-specific qualified machinery-safety engineering, verification and validation are external and not performed</x:v>
+        <x:v>Conceptual boundary and handoff exist; qualified machinery-safety/electrical verification and validation were not performed</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -31228,10 +31752,10 @@
         <x:v>Manifest independently verifies</x:v>
       </x:c>
       <x:c r="C23" s="6" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="D23" s="6" t="str">
-        <x:v>Published candidate f6e9f3b1e928a2e04d21913caac2547469b0f647 reproduced from GitHub with 425/425 manifest entries, zero discrepancies and final Git-clean assertion</x:v>
+        <x:v>Revision-G candidate manifest, final commit and post-push fresh-clone reproduction are pending release freeze</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -31242,7 +31766,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -31894,6 +32418,286 @@
         <x:v>Software-agent evidence</x:v>
       </x:c>
     </x:row>
+    <x:row r="33" ht="54" customHeight="1">
+      <x:c r="A33" s="6" t="str">
+        <x:v>DOC-G-001</x:v>
+      </x:c>
+      <x:c r="B33" s="6" t="str">
+        <x:v>Revision-G charter</x:v>
+      </x:c>
+      <x:c r="C33" s="6" t="str">
+        <x:v>00_project_control/revision_g_charter.md</x:v>
+      </x:c>
+      <x:c r="D33" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E33" s="6" t="str">
+        <x:v>Lead systems</x:v>
+      </x:c>
+      <x:c r="F33" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="54" customHeight="1">
+      <x:c r="A34" s="6" t="str">
+        <x:v>DOC-G-002</x:v>
+      </x:c>
+      <x:c r="B34" s="6" t="str">
+        <x:v>Revision-G gap matrix</x:v>
+      </x:c>
+      <x:c r="C34" s="6" t="str">
+        <x:v>00_project_control/revision_g_gap_matrix.csv</x:v>
+      </x:c>
+      <x:c r="D34" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E34" s="6" t="str">
+        <x:v>Lead systems</x:v>
+      </x:c>
+      <x:c r="F34" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="54" customHeight="1">
+      <x:c r="A35" s="6" t="str">
+        <x:v>DOC-G-003</x:v>
+      </x:c>
+      <x:c r="B35" s="6" t="str">
+        <x:v>Secure cloud architecture</x:v>
+      </x:c>
+      <x:c r="C35" s="6" t="str">
+        <x:v>cloud/architecture.md</x:v>
+      </x:c>
+      <x:c r="D35" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E35" s="6" t="str">
+        <x:v>Cloud security</x:v>
+      </x:c>
+      <x:c r="F35" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="54" customHeight="1">
+      <x:c r="A36" s="6" t="str">
+        <x:v>DOC-G-004</x:v>
+      </x:c>
+      <x:c r="B36" s="6" t="str">
+        <x:v>Cloud Terraform source</x:v>
+      </x:c>
+      <x:c r="C36" s="6" t="str">
+        <x:v>cloud/terraform/README.md</x:v>
+      </x:c>
+      <x:c r="D36" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E36" s="6" t="str">
+        <x:v>Cloud security</x:v>
+      </x:c>
+      <x:c r="F36" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="54" customHeight="1">
+      <x:c r="A37" s="6" t="str">
+        <x:v>DOC-G-005</x:v>
+      </x:c>
+      <x:c r="B37" s="6" t="str">
+        <x:v>Siemens native report</x:v>
+      </x:c>
+      <x:c r="C37" s="6" t="str">
+        <x:v>siemens_native/native_execution_report.md</x:v>
+      </x:c>
+      <x:c r="D37" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E37" s="6" t="str">
+        <x:v>Controls</x:v>
+      </x:c>
+      <x:c r="F37" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="54" customHeight="1">
+      <x:c r="A38" s="6" t="str">
+        <x:v>DOC-G-006</x:v>
+      </x:c>
+      <x:c r="B38" s="6" t="str">
+        <x:v>NVIDIA native report</x:v>
+      </x:c>
+      <x:c r="C38" s="6" t="str">
+        <x:v>nvidia_native/native_execution_report.md</x:v>
+      </x:c>
+      <x:c r="D38" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E38" s="6" t="str">
+        <x:v>Vision</x:v>
+      </x:c>
+      <x:c r="F38" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="54" customHeight="1">
+      <x:c r="A39" s="6" t="str">
+        <x:v>DOC-G-007</x:v>
+      </x:c>
+      <x:c r="B39" s="6" t="str">
+        <x:v>Commissioning package</x:v>
+      </x:c>
+      <x:c r="C39" s="6" t="str">
+        <x:v>commissioning/README.md</x:v>
+      </x:c>
+      <x:c r="D39" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E39" s="6" t="str">
+        <x:v>Commissioning</x:v>
+      </x:c>
+      <x:c r="F39" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="54" customHeight="1">
+      <x:c r="A40" s="6" t="str">
+        <x:v>DOC-G-008</x:v>
+      </x:c>
+      <x:c r="B40" s="6" t="str">
+        <x:v>Revision-G limitations</x:v>
+      </x:c>
+      <x:c r="C40" s="6" t="str">
+        <x:v>release/REVISION_G_KNOWN_LIMITATIONS.md</x:v>
+      </x:c>
+      <x:c r="D40" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E40" s="6" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="F40" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="54" customHeight="1">
+      <x:c r="A41" s="6" t="str">
+        <x:v>DOC-G-009</x:v>
+      </x:c>
+      <x:c r="B41" s="6" t="str">
+        <x:v>Revision-G evidence PDF</x:v>
+      </x:c>
+      <x:c r="C41" s="6" t="str">
+        <x:v>release/FC01_release_evidence.pdf</x:v>
+      </x:c>
+      <x:c r="D41" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E41" s="6" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="F41" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="54" customHeight="1">
+      <x:c r="A42" s="6" t="str">
+        <x:v>DOC-G-010</x:v>
+      </x:c>
+      <x:c r="B42" s="6" t="str">
+        <x:v>Revision-G engineering workbook</x:v>
+      </x:c>
+      <x:c r="C42" s="6" t="str">
+        <x:v>10_schedules/FC01_engineering_schedules.xlsx</x:v>
+      </x:c>
+      <x:c r="D42" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E42" s="6" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="F42" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="54" customHeight="1">
+      <x:c r="A43" s="6" t="str">
+        <x:v>DOC-G-011</x:v>
+      </x:c>
+      <x:c r="B43" s="6" t="str">
+        <x:v>Revision-G adversarial self-audit</x:v>
+      </x:c>
+      <x:c r="C43" s="6" t="str">
+        <x:v>14_qa/revision_g_audit_report.md</x:v>
+      </x:c>
+      <x:c r="D43" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E43" s="6" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="F43" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="54" customHeight="1">
+      <x:c r="A44" s="6" t="str">
+        <x:v>DOC-G-012</x:v>
+      </x:c>
+      <x:c r="B44" s="6" t="str">
+        <x:v>NVIDIA model/runtime evidence status</x:v>
+      </x:c>
+      <x:c r="C44" s="6" t="str">
+        <x:v>nvidia_native/model_card.md</x:v>
+      </x:c>
+      <x:c r="D44" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E44" s="6" t="str">
+        <x:v>Vision</x:v>
+      </x:c>
+      <x:c r="F44" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="54" customHeight="1">
+      <x:c r="A45" s="6" t="str">
+        <x:v>DOC-G-013</x:v>
+      </x:c>
+      <x:c r="B45" s="6" t="str">
+        <x:v>Qualified safety-review preparation</x:v>
+      </x:c>
+      <x:c r="C45" s="6" t="str">
+        <x:v>commissioning/qualified_review_handoff.md</x:v>
+      </x:c>
+      <x:c r="D45" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E45" s="6" t="str">
+        <x:v>Safety boundary</x:v>
+      </x:c>
+      <x:c r="F45" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="54" customHeight="1">
+      <x:c r="A46" s="6" t="str">
+        <x:v>DOC-G-014</x:v>
+      </x:c>
+      <x:c r="B46" s="6" t="str">
+        <x:v>Cloud plan status</x:v>
+      </x:c>
+      <x:c r="C46" s="6" t="str">
+        <x:v>cloud/plan_status.md</x:v>
+      </x:c>
+      <x:c r="D46" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E46" s="6" t="str">
+        <x:v>Cloud security</x:v>
+      </x:c>
+      <x:c r="F46" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
@@ -31902,7 +32706,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -31939,7 +32743,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="24" t="str">
-        <x:v>FICTIONAL ENGINEERING PROJECT - NOT FOR CONSTRUCTION | Revision F | NVIDIA implementation-readiness release candidate</x:v>
+        <x:v>FICTIONAL ENGINEERING PROJECT - NOT FOR CONSTRUCTION | Revision G | cloud-ready and native-execution-ready release candidate</x:v>
       </x:c>
       <x:c r="B3" s="24"/>
       <x:c r="C3" s="24"/>
@@ -31951,7 +32755,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="30" t="str">
-        <x:v>CONCEPTUAL SAFETY ARCHITECTURE - REQUIRES PROJECT-SPECIFIC RISK ASSESSMENT, DESIGN, VERIFICATION AND VALIDATION BY A QUALIFIED MACHINERY-SAFETY ENGINEER. NO PERFORMANCE LEVEL, SIL, CATEGORY, CE CONFORMITY OR REGULATORY COMPLIANCE IS CLAIMED.</x:v>
+        <x:v>CONCEPTUAL SAFETY ARCHITECTURE - REQUIRES PROJECT-SPECIFIC RISK ASSESSMENT, DESIGN, VERIFICATION AND VALIDATION BY A QUALIFIED MACHINERY-SAFETY ENGINEER. NO PERFORMANCE LEVEL, SIL, CATEGORY, CE/UKCA CONFORMITY OR REGULATORY COMPLIANCE IS CLAIMED.</x:v>
       </x:c>
       <x:c r="B4" s="30"/>
       <x:c r="C4" s="30"/>
@@ -31985,7 +32789,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="D6" s="46" t="str">
-        <x:v>Revision F includes a source-tested 47-node fail-closed PLC/AI contract, production-structured edge and dataset tooling, 28 structured behavioral vision fault injections, a controlled electrical delta, secure local asyncua integration and inherited native CAD/QET evidence. The behavioral model is software-only evidence, not PLCSIM, HIL or physical testing. THE NVIDIA VISION SUBSYSTEM IS NON-SAFETY-RELATED AND MUST NOT BE USED AS THE SOLE MEANS OF PERSONNEL PROTECTION, SAFE STOP, GUARD MONITORING OR HAZARDOUS-MOTION CONTROL. Native Siemens, real dataset/model, target runtime, site electrical, FAT/SAT, qualified safety and physical commissioning remain blocked or open exactly as listed.</x:v>
+        <x:v>Revision G preserves the source-tested 47-node fail-closed PLC/AI contract, secure local asyncua integration, 28 structured behavioral fault injections and inherited native CAD/QET evidence. It adds disabled-by-default cloud infrastructure, actual Siemens/NVIDIA inventory, exact external handoffs, data/model execution scaffolding and blank commissioning records. The evidence is software/laboratory only: no cloud apply, TIA/WinCC/Startdrive/PLCSIM compile, representative dataset, trained model, target runtime, physical test or qualified approval exists. THE NVIDIA VISION SUBSYSTEM IS NON-SAFETY-RELATED AND MUST NOT COMMAND HAZARDOUS MOTION OR BYPASS PLC INTERLOCKS.</x:v>
       </x:c>
       <x:c r="E6" s="46"/>
       <x:c r="F6" s="46"/>
@@ -32082,7 +32886,7 @@
       </x:c>
       <x:c r="B13" t="n">
         <x:f>COUNTIF('Acceptance Gates'!C2:C100,"PASS")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D13" s="46"/>
       <x:c r="E13" s="46"/>
@@ -32096,7 +32900,7 @@
       </x:c>
       <x:c r="B14" t="n">
         <x:f>COUNTIF('Acceptance Gates'!C2:C100,"PARTIAL")</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D14" s="46"/>
       <x:c r="E14" s="46"/>

</xml_diff>

<commit_message>
docs: attest Revision G published-candidate reproduction
</commit_message>
<xml_diff>
--- a/10_schedules/FC01_engineering_schedules.xlsx
+++ b/10_schedules/FC01_engineering_schedules.xlsx
@@ -584,8 +584,8 @@
 </file>
 
 <file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="DocumentRegisterTable" displayName="DocumentRegisterTable" ref="A1:F46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F46"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="DocumentRegisterTable" displayName="DocumentRegisterTable" ref="A1:F47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F47"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="document_id"/>
     <x:tableColumn id="2" name="title"/>
@@ -31752,10 +31752,10 @@
         <x:v>Manifest independently verifies</x:v>
       </x:c>
       <x:c r="C23" s="6" t="str">
-        <x:v>PARTIAL</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="D23" s="6" t="str">
-        <x:v>Revision-G candidate manifest, final commit and post-push fresh-clone reproduction are pending release freeze</x:v>
+        <x:v>Published candidate 38ab54deace5e6b71479bb4a347cd39c0233f37d reproduced from a fresh GitHub clone: manifest 504/504, zero discrepancies; see DOC-G-015</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -32695,6 +32695,26 @@
         <x:v>Cloud security</x:v>
       </x:c>
       <x:c r="F46" s="6" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="54" customHeight="1">
+      <x:c r="A47" s="6" t="str">
+        <x:v>DOC-G-015</x:v>
+      </x:c>
+      <x:c r="B47" s="6" t="str">
+        <x:v>Revision-G post-push reproduction</x:v>
+      </x:c>
+      <x:c r="C47" s="6" t="str">
+        <x:v>14_qa/revision_g_post_push_reproduction.md</x:v>
+      </x:c>
+      <x:c r="D47" s="6" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="E47" s="6" t="str">
+        <x:v>Configuration management</x:v>
+      </x:c>
+      <x:c r="F47" s="6" t="str">
         <x:v>Controlled</x:v>
       </x:c>
     </x:row>
@@ -32886,7 +32906,7 @@
       </x:c>
       <x:c r="B13" t="n">
         <x:f>COUNTIF('Acceptance Gates'!C2:C100,"PASS")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D13" s="46"/>
       <x:c r="E13" s="46"/>
@@ -32900,7 +32920,7 @@
       </x:c>
       <x:c r="B14" t="n">
         <x:f>COUNTIF('Acceptance Gates'!C2:C100,"PARTIAL")</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D14" s="46"/>
       <x:c r="E14" s="46"/>

</xml_diff>